<commit_message>
refactor: melhora roteiro de abordagem fria e adiciona resposta para casos positivos
</commit_message>
<xml_diff>
--- a/Prospecção/Leads_LashDesigner_Goiania.xlsx
+++ b/Prospecção/Leads_LashDesigner_Goiania.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M41"/>
+  <dimension ref="A1:N41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -481,15 +481,20 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Abordagem_WhatsApp</t>
+          <t>Abordagem_Inicial_WhatsApp</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
+          <t>Resposta_Se_Responder_SIM</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
           <t>Endereço</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Link_GoogleMaps</t>
         </is>
@@ -540,18 +545,24 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Oii Edivania, tudo bem? 👋 Vi o perfil de excelência do seu estúdio no Setor Central no Google (265 avaliações no Google! ⭐) e achei seu trabalho impecável.
-Percebi que muitas clientes aí em Goiânia ficam em dúvida sobre qual técnica escolher (Fio a Fio, Volume Russo, Brasileiro, Lash Lifting) ou sobre manutenções e valores antes de agendar.
-Desenvolvemos o *LashMenu*, um catálogo digital interativo feito sob medida para Lash Designers enviar pelo WhatsApp e colocar na Bio do Instagram. Ele organiza seus procedimentos, tabela de preços e orientações pós-procedimento em um só link profissional, acelerando o agendamento de clientes.
-Posso te enviar uma demonstração gratuita que montamos para o seu estúdio dar uma olhada rápida?</t>
+          <t>Oii Edivania, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
+Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
+          <t>Que ótimo Edivania! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
           <t>Av. Anhanguera, 5389 - St. Central, Goiânia - GO, 74043-010, Brasil</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Curso%20Extens%C3%A3o%20de%20c%C3%ADlios%20-%20Studio%20Edivania%20Paiva%20Extens%C3%A3o%20de%20c%C3%ADlios%20Goi%C3%A2nia&amp;query_place_id=ChIJNcJRVe7xXpMRegJRirWTQ3Q</t>
         </is>
@@ -602,18 +613,24 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Oii Layfer, tudo bem? 👋 Vi o perfil de excelência do seu estúdio no Alto da Glória no Google (228 avaliações no Google! ⭐) e achei seu trabalho impecável.
-Percebi que muitas clientes aí em Goiânia ficam em dúvida sobre qual técnica escolher (Fio a Fio, Volume Russo, Brasileiro, Lash Lifting) ou sobre manutenções e valores antes de agendar.
-Desenvolvemos o *LashMenu*, um catálogo digital interativo feito sob medida para Lash Designers enviar pelo WhatsApp e colocar na Bio do Instagram. Ele organiza seus procedimentos, tabela de preços e orientações pós-procedimento em um só link profissional, acelerando o agendamento de clientes.
-Posso te enviar uma demonstração gratuita que montamos para o seu estúdio dar uma olhada rápida?</t>
+          <t>Oii Layfer, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
+Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
+          <t>Que ótimo Layfer! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
           <t>Av. São João esq. c/ Rua Vitoria, Qd. 9, Lt. 11, Alto da Glória Sala 301., 3º Andar - Alto da Glória, Goiânia - GO, 74815-745, Brasil</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Studio%20Layfer%2C%20C%C3%ADlios%2C%20Micropigmenta%C3%A7%C3%A3o%20e%20Est%C3%A9tica%20-%20St.%20Alto%20da%20Gl%C3%B3ria&amp;query_place_id=ChIJzxi2-6PxXpMRk_q1l5AoAD4</t>
         </is>
@@ -660,18 +677,24 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Oii Larissa, tudo bem? 👋 Vi o perfil de excelência do seu estúdio no Setor Bueno no Google (117 avaliações no Google! ⭐) e achei seu trabalho impecável.
-Percebi que muitas clientes aí em Goiânia ficam em dúvida sobre qual técnica escolher (Fio a Fio, Volume Russo, Brasileiro, Lash Lifting) ou sobre manutenções e valores antes de agendar.
-Desenvolvemos o *LashMenu*, um catálogo digital interativo feito sob medida para Lash Designers enviar pelo WhatsApp e colocar na Bio do Instagram. Ele organiza seus procedimentos, tabela de preços e orientações pós-procedimento em um só link profissional, acelerando o agendamento de clientes.
-Posso te enviar uma demonstração gratuita que montamos para o seu estúdio dar uma olhada rápida?</t>
+          <t>Oii Larissa, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
+Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
+          <t>Que ótimo Larissa! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
           <t>R. T 1-A, 63 - St. Bueno, Goiânia - GO, 74210-330, Brasil</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Studio%20Larissa%20Lobo.%20Especializado%20em%20sobrancelhas%2C%20c%C3%ADlios%20e%20est%C3%A9tica.&amp;query_place_id=ChIJjchOyjzxXpMRxFD2HiV89GI</t>
         </is>
@@ -718,18 +741,24 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Oii Leticia, tudo bem? 👋 Vi o perfil de excelência do seu estúdio no Setor Bueno no Google (83 avaliações no Google! ⭐) e achei seu trabalho impecável.
-Percebi que muitas clientes aí em Goiânia ficam em dúvida sobre qual técnica escolher (Fio a Fio, Volume Russo, Brasileiro, Lash Lifting) ou sobre manutenções e valores antes de agendar.
-Desenvolvemos o *LashMenu*, um catálogo digital interativo feito sob medida para Lash Designers enviar pelo WhatsApp e colocar na Bio do Instagram. Ele organiza seus procedimentos, tabela de preços e orientações pós-procedimento em um só link profissional, acelerando o agendamento de clientes.
-Posso te enviar uma demonstração gratuita que montamos para o seu estúdio dar uma olhada rápida?</t>
+          <t>Oii Leticia, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
+Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
+          <t>Que ótimo Leticia! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
           <t>Av. T-15, 1380 - St. Bueno, Goiânia - GO, 74230-010, Brasil</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Extens%C3%A3o%20de%20c%C3%ADlios%20Goiania%20-%20Studio%20Leticia%20Santana%20Lash%20Design&amp;query_place_id=ChIJG9x9B23xXpMRznt7moxKXfw</t>
         </is>
@@ -776,18 +805,24 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Oii Poliana, tudo bem? 👋 Vi o perfil de excelência do seu estúdio no Setor Marista no Google (57 avaliações no Google! ⭐) e achei seu trabalho impecável.
-Percebi que muitas clientes aí em Goiânia ficam em dúvida sobre qual técnica escolher (Fio a Fio, Volume Russo, Brasileiro, Lash Lifting) ou sobre manutenções e valores antes de agendar.
-Desenvolvemos o *LashMenu*, um catálogo digital interativo feito sob medida para Lash Designers enviar pelo WhatsApp e colocar na Bio do Instagram. Ele organiza seus procedimentos, tabela de preços e orientações pós-procedimento em um só link profissional, acelerando o agendamento de clientes.
-Posso te enviar uma demonstração gratuita que montamos para o seu estúdio dar uma olhada rápida?</t>
+          <t>Oii Poliana, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
+Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
+          <t>Que ótimo Poliana! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
           <t>R. 1137, 225 - QD; 243 LOTE 2 - St. Marista, Goiânia - GO, 74180-160, Brasil</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Extens%C3%A3o%20de%20c%C3%ADlios%20By%20Poliana%20Souza&amp;query_place_id=ChIJl_ZyRl_xXpMRoMv8tRv3jHo</t>
         </is>
@@ -838,18 +873,24 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Oii Tanielly, tudo bem? 👋 Vi o perfil de excelência do seu estúdio no Alto da Glória no Google (53 avaliações no Google! ⭐) e achei seu trabalho impecável.
-Percebi que muitas clientes aí em Goiânia ficam em dúvida sobre qual técnica escolher (Fio a Fio, Volume Russo, Brasileiro, Lash Lifting) ou sobre manutenções e valores antes de agendar.
-Desenvolvemos o *LashMenu*, um catálogo digital interativo feito sob medida para Lash Designers enviar pelo WhatsApp e colocar na Bio do Instagram. Ele organiza seus procedimentos, tabela de preços e orientações pós-procedimento em um só link profissional, acelerando o agendamento de clientes.
-Posso te enviar uma demonstração gratuita que montamos para o seu estúdio dar uma olhada rápida?</t>
+          <t>Oii Tanielly, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
+Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
+          <t>Que ótimo Tanielly! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
           <t>R. São Luís, 364 - Alto da Glória, Goiânia - GO, 74815-755, Brasil</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Tanielly%20Duarte%20Studio%20Beauty&amp;query_place_id=ChIJw-k52L7xXpMRSfLrH3GEy1E</t>
         </is>
@@ -896,18 +937,24 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Oii Serena, tudo bem? 👋 Vi o perfil de excelência do seu estúdio no Jardim Goiás no Google (55 avaliações no Google! ⭐) e achei seu trabalho impecável.
-Percebi que muitas clientes aí em Goiânia ficam em dúvida sobre qual técnica escolher (Fio a Fio, Volume Russo, Brasileiro, Lash Lifting) ou sobre manutenções e valores antes de agendar.
-Desenvolvemos o *LashMenu*, um catálogo digital interativo feito sob medida para Lash Designers enviar pelo WhatsApp e colocar na Bio do Instagram. Ele organiza seus procedimentos, tabela de preços e orientações pós-procedimento em um só link profissional, acelerando o agendamento de clientes.
-Posso te enviar uma demonstração gratuita que montamos para o seu estúdio dar uma olhada rápida?</t>
+          <t>Oii Serena, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
+Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
+          <t>Que ótimo Serena! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
           <t>Edifício Trend Office - R. 72, 325 - Sl 1101 - Jardim Goiás, Goiânia - GO, 74805-480, Brasil</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Serena%20Beauty&amp;query_place_id=ChIJ30V_nJLzXpMRZxr4KhUVXi8</t>
         </is>
@@ -958,18 +1005,24 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Oii Cinthya, tudo bem? 👋 Vi o perfil de excelência do seu estúdio no Setor Bela Vista no Google (74 avaliações no Google! ⭐) e achei seu trabalho impecável.
-Percebi que muitas clientes aí em Goiânia ficam em dúvida sobre qual técnica escolher (Fio a Fio, Volume Russo, Brasileiro, Lash Lifting) ou sobre manutenções e valores antes de agendar.
-Desenvolvemos o *LashMenu*, um catálogo digital interativo feito sob medida para Lash Designers enviar pelo WhatsApp e colocar na Bio do Instagram. Ele organiza seus procedimentos, tabela de preços e orientações pós-procedimento em um só link profissional, acelerando o agendamento de clientes.
-Posso te enviar uma demonstração gratuita que montamos para o seu estúdio dar uma olhada rápida?</t>
+          <t>Oii Cinthya, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
+Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
+          <t>Que ótimo Cinthya! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
           <t>Comercial das acácias - Alameda Couto Magalhães, 755 - qd S-28 lt 4 sala 201 - St. Bela Vista, Goiânia - GO, 74823-410, Brasil</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Studio%20Cinthya%20Montanini%20Goi%C3%A2nia%2C%20Extens%C3%A3o%20de%20C%C3%ADlios%2C%20Micropigmenta%C3%A7%C3%A3o%20de%20Sobrancelha%2C%20Labial%20e%20alongamento%20de%20unha&amp;query_place_id=ChIJGzUau7jxXpMRuco3wD_9oYU</t>
         </is>
@@ -1020,18 +1073,24 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Oii Design, tudo bem? 👋 Vi o perfil de excelência do seu estúdio no Setor Sul no Google (73 avaliações no Google! ⭐) e achei seu trabalho impecável.
-Percebi que muitas clientes aí em Goiânia ficam em dúvida sobre qual técnica escolher (Fio a Fio, Volume Russo, Brasileiro, Lash Lifting) ou sobre manutenções e valores antes de agendar.
-Desenvolvemos o *LashMenu*, um catálogo digital interativo feito sob medida para Lash Designers enviar pelo WhatsApp e colocar na Bio do Instagram. Ele organiza seus procedimentos, tabela de preços e orientações pós-procedimento em um só link profissional, acelerando o agendamento de clientes.
-Posso te enviar uma demonstração gratuita que montamos para o seu estúdio dar uma olhada rápida?</t>
+          <t>Oii Design, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
+Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
+          <t>Que ótimo Design! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
           <t>Rua 131 Q Area, 342 - St. Sul, Goiânia - GO, 74093-200, Brasil</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Design%20de%20Sobrancelhas%20e%20brow%20lamination%20Goi%C3%A2nia%20-%20Milenne%20Beauty%20Organiq&amp;query_place_id=ChIJKSdJ9xXxXpMR2i-K-1q6l5w</t>
         </is>
@@ -1082,18 +1141,24 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Oii Design, tudo bem? 👋 Vi o perfil de excelência do seu estúdio no Setor Leste Universitário no Google (68 avaliações no Google! ⭐) e achei seu trabalho impecável.
-Percebi que muitas clientes aí em Goiânia ficam em dúvida sobre qual técnica escolher (Fio a Fio, Volume Russo, Brasileiro, Lash Lifting) ou sobre manutenções e valores antes de agendar.
-Desenvolvemos o *LashMenu*, um catálogo digital interativo feito sob medida para Lash Designers enviar pelo WhatsApp e colocar na Bio do Instagram. Ele organiza seus procedimentos, tabela de preços e orientações pós-procedimento em um só link profissional, acelerando o agendamento de clientes.
-Posso te enviar uma demonstração gratuita que montamos para o seu estúdio dar uma olhada rápida?</t>
+          <t>Oii Design, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
+Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
+          <t>Que ótimo Design! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
           <t>R. 217, 930 - Setor Leste Universitário, Goiânia - GO, 74603-090, Brasil</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Extens%C3%A3o%20de%20C%C3%ADlios%20e%20Design%20de%20Sobrancelhas%20%7C%20Studio%20Brunna%20Lima%20Beauty%20Goi%C3%A2nia&amp;query_place_id=ChIJr9nEaLHzXpMR93NBR10NBeY</t>
         </is>
@@ -1144,18 +1209,24 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Oii Bella, tudo bem? 👋 Vi o perfil de excelência do seu estúdio no Setor Negrão de Lima no Google (52 avaliações no Google! ⭐) e achei seu trabalho impecável.
-Percebi que muitas clientes aí em Goiânia ficam em dúvida sobre qual técnica escolher (Fio a Fio, Volume Russo, Brasileiro, Lash Lifting) ou sobre manutenções e valores antes de agendar.
-Desenvolvemos o *LashMenu*, um catálogo digital interativo feito sob medida para Lash Designers enviar pelo WhatsApp e colocar na Bio do Instagram. Ele organiza seus procedimentos, tabela de preços e orientações pós-procedimento em um só link profissional, acelerando o agendamento de clientes.
-Posso te enviar uma demonstração gratuita que montamos para o seu estúdio dar uma olhada rápida?</t>
+          <t>Oii Bella, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
+Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
+          <t>Que ótimo Bella! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
           <t>R. Dona Mariquinha, Qd 21 - Lt 26 sala 01 - Setor Negrão de Lima, Goiânia - GO, 74650-130, Brasil</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="N12" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Bella%20C%C3%ADlios%20e%20sobrancelhas&amp;query_place_id=ChIJqcYJEjXyXpMRtnQQ3biylr4</t>
         </is>
@@ -1206,18 +1277,24 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Oii Maria, tudo bem? 👋 Vi o perfil de excelência do seu estúdio no Parque Atheneu no Google (48 avaliações no Google! ⭐) e achei seu trabalho impecável.
-Percebi que muitas clientes aí em Goiânia ficam em dúvida sobre qual técnica escolher (Fio a Fio, Volume Russo, Brasileiro, Lash Lifting) ou sobre manutenções e valores antes de agendar.
-Desenvolvemos o *LashMenu*, um catálogo digital interativo feito sob medida para Lash Designers enviar pelo WhatsApp e colocar na Bio do Instagram. Ele organiza seus procedimentos, tabela de preços e orientações pós-procedimento em um só link profissional, acelerando o agendamento de clientes.
-Posso te enviar uma demonstração gratuita que montamos para o seu estúdio dar uma olhada rápida?</t>
+          <t>Oii Maria, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
+Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
+          <t>Que ótimo Maria! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
           <t>R. 3, lote 8 - unidade 103 - Parque Atheneu, Goiânia - GO, 74893-130, Brasil</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="N13" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Studio%20Maria%20Eug%C3%AAnia%20Sobrancelhas&amp;query_place_id=ChIJU43d51L1XpMRs5E5kKLMxX0</t>
         </is>
@@ -1268,18 +1345,24 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Oii Mariane, tudo bem? 👋 Vi o perfil de excelência do seu estúdio no Parque Atheneu no Google (43 avaliações no Google! ⭐) e achei seu trabalho impecável.
-Percebi que muitas clientes aí em Goiânia ficam em dúvida sobre qual técnica escolher (Fio a Fio, Volume Russo, Brasileiro, Lash Lifting) ou sobre manutenções e valores antes de agendar.
-Desenvolvemos o *LashMenu*, um catálogo digital interativo feito sob medida para Lash Designers enviar pelo WhatsApp e colocar na Bio do Instagram. Ele organiza seus procedimentos, tabela de preços e orientações pós-procedimento em um só link profissional, acelerando o agendamento de clientes.
-Posso te enviar uma demonstração gratuita que montamos para o seu estúdio dar uma olhada rápida?</t>
+          <t>Oii Mariane, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
+Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
+          <t>Que ótimo Mariane! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
           <t>R. Quinze, 47 - Und 201 - Parque Atheneu, Goiânia - GO, 74890-230, Brasil</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
+      <c r="N14" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Mariane%20Moreno%20Sobrancelhas&amp;query_place_id=ChIJX1H2g17lXpMRgNeUw_-gzZw</t>
         </is>
@@ -1330,18 +1413,24 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Oii Isabela, tudo bem? 👋 Vi o perfil de excelência do seu estúdio no Vila Redencao no Google (31 avaliações no Google! ⭐) e achei seu trabalho impecável.
-Percebi que muitas clientes aí em Goiânia ficam em dúvida sobre qual técnica escolher (Fio a Fio, Volume Russo, Brasileiro, Lash Lifting) ou sobre manutenções e valores antes de agendar.
-Desenvolvemos o *LashMenu*, um catálogo digital interativo feito sob medida para Lash Designers enviar pelo WhatsApp e colocar na Bio do Instagram. Ele organiza seus procedimentos, tabela de preços e orientações pós-procedimento em um só link profissional, acelerando o agendamento de clientes.
-Posso te enviar uma demonstração gratuita que montamos para o seu estúdio dar uma olhada rápida?</t>
+          <t>Oii Isabela, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
+Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
+          <t>Que ótimo Isabela! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
           <t>Av. 2ª Radial, Qd. 70 - Lt. 06 Sala 2 - Vila Redencao, Goiânia - GO, 74850-040, Brasil</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="N15" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Studio%20Isabela%20Souza%20%7C%20C%C3%ADlios%20e%20Sobrancelhas%20em%20Goi%C3%A2nia&amp;query_place_id=ChIJ6_FUKYnxXpMRZl7o8vNiDJE</t>
         </is>
@@ -1392,18 +1481,24 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Oii Déborah, tudo bem? 👋 Vi o perfil de excelência do seu estúdio no Nova Suiça no Google (27 avaliações no Google! ⭐) e achei seu trabalho impecável.
-Percebi que muitas clientes aí em Goiânia ficam em dúvida sobre qual técnica escolher (Fio a Fio, Volume Russo, Brasileiro, Lash Lifting) ou sobre manutenções e valores antes de agendar.
-Desenvolvemos o *LashMenu*, um catálogo digital interativo feito sob medida para Lash Designers enviar pelo WhatsApp e colocar na Bio do Instagram. Ele organiza seus procedimentos, tabela de preços e orientações pós-procedimento em um só link profissional, acelerando o agendamento de clientes.
-Posso te enviar uma demonstração gratuita que montamos para o seu estúdio dar uma olhada rápida?</t>
+          <t>Oii Déborah, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
+Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
+          <t>Que ótimo Déborah! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
           <t>Sobrancelha Natural, Cílios, Design, Henna Cílios em - R. C-252, N° 1141 - QD 604, LT 11 - Nova Suiça, Goiânia - GO, 74280-160, Brasil</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr">
+      <c r="N16" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=D%C3%A9borah%20Alvarenga%20Beauty%20-%20C%C3%ADlios%20Goi%C3%A2nia%20%2F%20Sobrancelha%20Natural%20%2F%20C%C3%ADlios&amp;query_place_id=ChIJl9chJ-nxXpMRqLdSKfOsPEI</t>
         </is>
@@ -1454,18 +1549,24 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Oii Yara, tudo bem? 👋 Vi o perfil de excelência do seu estúdio em Goiânia no Google (23 avaliações no Google! ⭐) e achei seu trabalho impecável.
-Percebi que muitas clientes aí em Goiânia ficam em dúvida sobre qual técnica escolher (Fio a Fio, Volume Russo, Brasileiro, Lash Lifting) ou sobre manutenções e valores antes de agendar.
-Desenvolvemos o *LashMenu*, um catálogo digital interativo feito sob medida para Lash Designers enviar pelo WhatsApp e colocar na Bio do Instagram. Ele organiza seus procedimentos, tabela de preços e orientações pós-procedimento em um só link profissional, acelerando o agendamento de clientes.
-Posso te enviar uma demonstração gratuita que montamos para o seu estúdio dar uma olhada rápida?</t>
+          <t>Oii Yara, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
+Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
+          <t>Que ótimo Yara! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
           <t>R. Poe. Joaquim Bonifácio - Goiânia, GO, 74770-410, Brasil</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr">
+      <c r="N17" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Yara%20Ferreira%20Lash%20Designer%20-%20Extens%C3%A3o%20de%20C%C3%ADlios&amp;query_place_id=ChIJyxTL8p7vXpMR1pVLBLcrUEg</t>
         </is>
@@ -1512,18 +1613,24 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Oii Kathellem, tudo bem? 👋 Vi o perfil de excelência do seu estúdio no Setor Leste Universitário no Google (22 avaliações no Google! ⭐) e achei seu trabalho impecável.
-Percebi que muitas clientes aí em Goiânia ficam em dúvida sobre qual técnica escolher (Fio a Fio, Volume Russo, Brasileiro, Lash Lifting) ou sobre manutenções e valores antes de agendar.
-Desenvolvemos o *LashMenu*, um catálogo digital interativo feito sob medida para Lash Designers enviar pelo WhatsApp e colocar na Bio do Instagram. Ele organiza seus procedimentos, tabela de preços e orientações pós-procedimento em um só link profissional, acelerando o agendamento de clientes.
-Posso te enviar uma demonstração gratuita que montamos para o seu estúdio dar uma olhada rápida?</t>
+          <t>Oii Kathellem, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
+Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
+          <t>Que ótimo Kathellem! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
           <t>R. 233, 1483 - Qd 78 Lt 12 - Setor Leste Universitário, Goiânia - GO, 74605-120, Brasil</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr">
+      <c r="N18" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Studio%20Kathellem%20lima%20-%20Lash%20Designer%20(Extens%C3%A3o%20de%20c%C3%ADlios)-%20Designer%20de%20sobrancelha%20-%20maquiagem-Depila%C3%A7%C3%A3o&amp;query_place_id=ChIJlQQGMQzxXpMRzMyTFfdm_pU</t>
         </is>
@@ -1570,18 +1677,24 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Oii Lollys, tudo bem? 👋 Vi o perfil de excelência do seu estúdio no Nova Suiça no Google (41 avaliações no Google! ⭐) e achei seu trabalho impecável.
-Percebi que muitas clientes aí em Goiânia ficam em dúvida sobre qual técnica escolher (Fio a Fio, Volume Russo, Brasileiro, Lash Lifting) ou sobre manutenções e valores antes de agendar.
-Desenvolvemos o *LashMenu*, um catálogo digital interativo feito sob medida para Lash Designers enviar pelo WhatsApp e colocar na Bio do Instagram. Ele organiza seus procedimentos, tabela de preços e orientações pós-procedimento em um só link profissional, acelerando o agendamento de clientes.
-Posso te enviar uma demonstração gratuita que montamos para o seu estúdio dar uma olhada rápida?</t>
+          <t>Oii Lollys, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
+Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
+          <t>Que ótimo Lollys! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
           <t>Av. C-255, 271 - Nova Suiça, Goiânia - GO, 74280-010, Brasil</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr">
+      <c r="N19" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Studio%20Lollys%20Cilios&amp;query_place_id=ChIJGye0ibH2XpMRF8fxewDzYv4</t>
         </is>
@@ -1624,18 +1737,24 @@
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Oii Ariana, tudo bem? 👋 Vi o perfil de excelência do seu estúdio no Leste Vila Nova no Google (32 avaliações no Google! ⭐) e achei seu trabalho impecável.
-Percebi que muitas clientes aí em Goiânia ficam em dúvida sobre qual técnica escolher (Fio a Fio, Volume Russo, Brasileiro, Lash Lifting) ou sobre manutenções e valores antes de agendar.
-Desenvolvemos o *LashMenu*, um catálogo digital interativo feito sob medida para Lash Designers enviar pelo WhatsApp e colocar na Bio do Instagram. Ele organiza seus procedimentos, tabela de preços e orientações pós-procedimento em um só link profissional, acelerando o agendamento de clientes.
-Posso te enviar uma demonstração gratuita que montamos para o seu estúdio dar uma olhada rápida?</t>
+          <t>Oii Ariana, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
+Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
+          <t>Que ótimo Ariana! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
           <t>R. 209-A, 1405 - Leste Vila Nova, Goiânia - GO, 74645-210, Brasil</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr">
+      <c r="N20" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=EXTENS%C3%83O%20DE%20C%C3%8DLIOS%20GOI%C3%82NIA-%20ARIANA&amp;query_place_id=ChIJOU-jj6jzXpMROoQLtO7YqUw</t>
         </is>
@@ -1678,18 +1797,24 @@
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Oii Design, tudo bem? 👋 Vi o perfil de excelência do seu estúdio no Setor Sul no Google (245 avaliações no Google! ⭐) e achei seu trabalho impecável.
-Percebi que muitas clientes aí em Goiânia ficam em dúvida sobre qual técnica escolher (Fio a Fio, Volume Russo, Brasileiro, Lash Lifting) ou sobre manutenções e valores antes de agendar.
-Desenvolvemos o *LashMenu*, um catálogo digital interativo feito sob medida para Lash Designers enviar pelo WhatsApp e colocar na Bio do Instagram. Ele organiza seus procedimentos, tabela de preços e orientações pós-procedimento em um só link profissional, acelerando o agendamento de clientes.
-Posso te enviar uma demonstração gratuita que montamos para o seu estúdio dar uma olhada rápida?</t>
+          <t>Oii Design, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
+Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
+          <t>Que ótimo Design! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
           <t>Qd F37 28, R. 88-D, 286 - St. Sul, Goiânia - GO, 74085-115, Brasil</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr">
+      <c r="N21" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Sobrancelhas%20Design&amp;query_place_id=ChIJv6BTMnPxXpMRSTgLft6uVY4</t>
         </is>
@@ -1740,18 +1865,24 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Oii Elaíne, tudo bem? 👋 Vi o perfil de excelência do seu estúdio no Parque das Amendoeiras no Google (19 avaliações no Google! ⭐) e achei seu trabalho impecável.
-Percebi que muitas clientes aí em Goiânia ficam em dúvida sobre qual técnica escolher (Fio a Fio, Volume Russo, Brasileiro, Lash Lifting) ou sobre manutenções e valores antes de agendar.
-Desenvolvemos o *LashMenu*, um catálogo digital interativo feito sob medida para Lash Designers enviar pelo WhatsApp e colocar na Bio do Instagram. Ele organiza seus procedimentos, tabela de preços e orientações pós-procedimento em um só link profissional, acelerando o agendamento de clientes.
-Posso te enviar uma demonstração gratuita que montamos para o seu estúdio dar uma olhada rápida?</t>
+          <t>Oii Elaíne, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
+Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
+          <t>Que ótimo Elaíne! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
           <t>Av. Francisco Ludovíco de Almeida, qd35 lote17 - Parque das Amendoeiras, Goiânia - GO, 74780-440, Brasil</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr">
+      <c r="N22" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Ela%C3%ADne%20Nascimento%20Lashdesigner%20-%20Extens%C3%A3o%20de%20c%C3%ADlios%20e%20Designer%20de%20Sobrancelha%20em%20Goi%C3%A2nia&amp;query_place_id=ChIJB0t6XAztXpMRfyugbg31EHw</t>
         </is>
@@ -1798,18 +1929,24 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Oii Cílios, tudo bem? 👋 Vi o perfil de excelência do seu estúdio no Bairro Santa Rita no Google (16 avaliações no Google! ⭐) e achei seu trabalho impecável.
-Percebi que muitas clientes aí em Goiânia ficam em dúvida sobre qual técnica escolher (Fio a Fio, Volume Russo, Brasileiro, Lash Lifting) ou sobre manutenções e valores antes de agendar.
-Desenvolvemos o *LashMenu*, um catálogo digital interativo feito sob medida para Lash Designers enviar pelo WhatsApp e colocar na Bio do Instagram. Ele organiza seus procedimentos, tabela de preços e orientações pós-procedimento em um só link profissional, acelerando o agendamento de clientes.
-Posso te enviar uma demonstração gratuita que montamos para o seu estúdio dar uma olhada rápida?</t>
+          <t>Oii Cílios, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
+Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
+          <t>Que ótimo Cílios! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
           <t>R. João Luís, qd 07 - LT 07 - Bairro Santa Rita, Goiânia - GO, 74370-580, Brasil</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr">
+      <c r="N23" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Extens%C3%A3o%20de%20C%C3%ADlios%20-%20Studio%20de%20C%C3%ADlios%20Nayara&amp;query_place_id=ChIJG8ux-Ov3XpMRWf58BW9LZ5c</t>
         </is>
@@ -1860,18 +1997,24 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Oii Joana, tudo bem? 👋 Vi o perfil de excelência do seu estúdio no Residencial Paulo estrela no Google (16 avaliações no Google! ⭐) e achei seu trabalho impecável.
-Percebi que muitas clientes aí em Goiânia ficam em dúvida sobre qual técnica escolher (Fio a Fio, Volume Russo, Brasileiro, Lash Lifting) ou sobre manutenções e valores antes de agendar.
-Desenvolvemos o *LashMenu*, um catálogo digital interativo feito sob medida para Lash Designers enviar pelo WhatsApp e colocar na Bio do Instagram. Ele organiza seus procedimentos, tabela de preços e orientações pós-procedimento em um só link profissional, acelerando o agendamento de clientes.
-Posso te enviar uma demonstração gratuita que montamos para o seu estúdio dar uma olhada rápida?</t>
+          <t>Oii Joana, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
+Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
+          <t>Que ótimo Joana! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
           <t>R. 9, qd 09 lt 02 casa 1 - Residencial Paulo estrela, Goiânia - GO, 74786-444, Brasil</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr">
+      <c r="N24" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Joana%20Paiva%20studio&amp;query_place_id=ChIJJ3J5bgntXpMRud_xJ4tempE</t>
         </is>
@@ -1918,18 +2061,24 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Oii Cílios, tudo bem? 👋 Vi o perfil de excelência do seu estúdio no Crimeia Leste no Google (15 avaliações no Google! ⭐) e achei seu trabalho impecável.
-Percebi que muitas clientes aí em Goiânia ficam em dúvida sobre qual técnica escolher (Fio a Fio, Volume Russo, Brasileiro, Lash Lifting) ou sobre manutenções e valores antes de agendar.
-Desenvolvemos o *LashMenu*, um catálogo digital interativo feito sob medida para Lash Designers enviar pelo WhatsApp e colocar na Bio do Instagram. Ele organiza seus procedimentos, tabela de preços e orientações pós-procedimento em um só link profissional, acelerando o agendamento de clientes.
-Posso te enviar uma demonstração gratuita que montamos para o seu estúdio dar uma olhada rápida?</t>
+          <t>Oii Cílios, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
+Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
+          <t>Que ótimo Cílios! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
           <t>R. Gen. Braz Arantes, 129 - qd09 lt11 - Crimeia Leste, Goiânia - GO, 74660-210, Brasil</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr">
+      <c r="N25" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=C%C3%ADlios%20Showroom&amp;query_place_id=ChIJu0BGTGvzXpMRocxq8JKc-Sw</t>
         </is>
@@ -1976,18 +2125,24 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Oii Katyane, tudo bem? 👋 Vi o perfil de excelência do seu estúdio no Parque Atheneu no Google (11 avaliações no Google! ⭐) e achei seu trabalho impecável.
-Percebi que muitas clientes aí em Goiânia ficam em dúvida sobre qual técnica escolher (Fio a Fio, Volume Russo, Brasileiro, Lash Lifting) ou sobre manutenções e valores antes de agendar.
-Desenvolvemos o *LashMenu*, um catálogo digital interativo feito sob medida para Lash Designers enviar pelo WhatsApp e colocar na Bio do Instagram. Ele organiza seus procedimentos, tabela de preços e orientações pós-procedimento em um só link profissional, acelerando o agendamento de clientes.
-Posso te enviar uma demonstração gratuita que montamos para o seu estúdio dar uma olhada rápida?</t>
+          <t>Oii Katyane, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
+Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
+          <t>Que ótimo Katyane! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
           <t>Rua 2031, R. 1 Unidade 203 - Parque Atheneu, Goiânia - GO, 74890-700, Brasil</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr">
+      <c r="N26" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Studio%20Katyane%20Mendes&amp;query_place_id=ChIJDWwGdzblXpMRd3FPc_MqTIE</t>
         </is>
@@ -2030,18 +2185,24 @@
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Oii Vidal, tudo bem? 👋 Vi o perfil de excelência do seu estúdio no Parque Atheneu no Google (61 avaliações no Google! ⭐) e achei seu trabalho impecável.
-Percebi que muitas clientes aí em Goiânia ficam em dúvida sobre qual técnica escolher (Fio a Fio, Volume Russo, Brasileiro, Lash Lifting) ou sobre manutenções e valores antes de agendar.
-Desenvolvemos o *LashMenu*, um catálogo digital interativo feito sob medida para Lash Designers enviar pelo WhatsApp e colocar na Bio do Instagram. Ele organiza seus procedimentos, tabela de preços e orientações pós-procedimento em um só link profissional, acelerando o agendamento de clientes.
-Posso te enviar uma demonstração gratuita que montamos para o seu estúdio dar uma olhada rápida?</t>
+          <t>Oii Vidal, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
+Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
+          <t>Que ótimo Vidal! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
           <t>Rua 101 unid101, lote 2, Goiânia - GO, 74893-530, Brasil</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr">
+      <c r="N27" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Studio%20Vidal%20Priscila&amp;query_place_id=ChIJy5B_VJv7XpMRvSe-I9ZXO6M</t>
         </is>
@@ -2084,18 +2245,24 @@
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr">
         <is>
-          <t>Oii Crys, tudo bem? 👋 Vi o perfil de excelência do seu estúdio no Água Branca no Google (25 avaliações no Google! ⭐) e achei seu trabalho impecável.
-Percebi que muitas clientes aí em Goiânia ficam em dúvida sobre qual técnica escolher (Fio a Fio, Volume Russo, Brasileiro, Lash Lifting) ou sobre manutenções e valores antes de agendar.
-Desenvolvemos o *LashMenu*, um catálogo digital interativo feito sob medida para Lash Designers enviar pelo WhatsApp e colocar na Bio do Instagram. Ele organiza seus procedimentos, tabela de preços e orientações pós-procedimento em um só link profissional, acelerando o agendamento de clientes.
-Posso te enviar uma demonstração gratuita que montamos para o seu estúdio dar uma olhada rápida?</t>
+          <t>Oii Crys, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
+Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
+          <t>Que ótimo Crys! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
           <t>Av. F, quadra A - lote 04 - Setor - Água Branca, Goiânia - GO, 74730-320, Brasil</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr">
+      <c r="N28" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Crys%20Lohany%20Lashes&amp;query_place_id=ChIJE3PPbB7xXpMR8fpw2IcHaEo</t>
         </is>
@@ -2138,18 +2305,24 @@
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Oii Aliany, tudo bem? 👋 Vi o perfil de excelência do seu estúdio no Jardim Bela Vista no Google (24 avaliações no Google! ⭐) e achei seu trabalho impecável.
-Percebi que muitas clientes aí em Goiânia ficam em dúvida sobre qual técnica escolher (Fio a Fio, Volume Russo, Brasileiro, Lash Lifting) ou sobre manutenções e valores antes de agendar.
-Desenvolvemos o *LashMenu*, um catálogo digital interativo feito sob medida para Lash Designers enviar pelo WhatsApp e colocar na Bio do Instagram. Ele organiza seus procedimentos, tabela de preços e orientações pós-procedimento em um só link profissional, acelerando o agendamento de clientes.
-Posso te enviar uma demonstração gratuita que montamos para o seu estúdio dar uma olhada rápida?</t>
+          <t>Oii Aliany, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
+Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
+          <t>Que ótimo Aliany! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
           <t>Av. Bela Vista, qd i lt1 - Jardim Bela Vista, Goiânia - GO, 74863-050, Brasil</t>
         </is>
       </c>
-      <c r="M29" t="inlineStr">
+      <c r="N29" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Studio%20Aliany%20Mendes%20-%20Nail%20Designer&amp;query_place_id=ChIJkUJBKqrxXpMR6xxIrqyhBBg</t>
         </is>
@@ -2196,18 +2369,24 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Oii D'isanto, tudo bem? 👋 Vi o perfil de excelência do seu estúdio no Jardim Mariliza no Google ⭐ e achei seu trabalho impecável.
-Percebi que muitas clientes aí em Goiânia ficam em dúvida sobre qual técnica escolher (Fio a Fio, Volume Russo, Brasileiro, Lash Lifting) ou sobre manutenções e valores antes de agendar.
-Desenvolvemos o *LashMenu*, um catálogo digital interativo feito sob medida para Lash Designers enviar pelo WhatsApp e colocar na Bio do Instagram. Ele organiza seus procedimentos, tabela de preços e orientações pós-procedimento em um só link profissional, acelerando o agendamento de clientes.
-Posso te enviar uma demonstração gratuita que montamos para o seu estúdio dar uma olhada rápida?</t>
+          <t>Oii D'isanto, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
+Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
+          <t>Que ótimo D'isanto! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
           <t>R. Caraíba - Jardim Mariliza, Goiânia - GO, 74885-090, Brasil</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr">
+      <c r="N30" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=D'Isanto%20Brows%20%7C%20Design%20de%20Sobrancelhas%20%7C%20Brow%20Lamination%20%7C%20Lash%20Lifting&amp;query_place_id=ChIJURiAgEv7XpMRzE1r8meSquY</t>
         </is>
@@ -2258,18 +2437,24 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Oii Ynnaê, tudo bem? 👋 Vi o perfil de excelência do seu estúdio no Jardim das Aroeiras no Google ⭐ e achei seu trabalho impecável.
-Percebi que muitas clientes aí em Goiânia ficam em dúvida sobre qual técnica escolher (Fio a Fio, Volume Russo, Brasileiro, Lash Lifting) ou sobre manutenções e valores antes de agendar.
-Desenvolvemos o *LashMenu*, um catálogo digital interativo feito sob medida para Lash Designers enviar pelo WhatsApp e colocar na Bio do Instagram. Ele organiza seus procedimentos, tabela de preços e orientações pós-procedimento em um só link profissional, acelerando o agendamento de clientes.
-Posso te enviar uma demonstração gratuita que montamos para o seu estúdio dar uma olhada rápida?</t>
+          <t>Oii Ynnaê, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
+Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
+          <t>Que ótimo Ynnaê! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
           <t>R. JDA Dez, Quadra 07 lote 14 sala 01 - Jardim das Aroeiras, Goiânia - GO, 74770-550, Brasil</t>
         </is>
       </c>
-      <c r="M31" t="inlineStr">
+      <c r="N31" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Ynna%C3%AA%20Uch%C3%B4a%20Lash%20Design%20Micropigmentadora&amp;query_place_id=ChIJiTtbqZfvXpMRIO3w6gfFvF8</t>
         </is>
@@ -2320,18 +2505,24 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>Oii Tiffany, tudo bem? 👋 Vi o perfil de excelência do seu estúdio no Dom Fernando II no Google ⭐ e achei seu trabalho impecável.
-Percebi que muitas clientes aí em Goiânia ficam em dúvida sobre qual técnica escolher (Fio a Fio, Volume Russo, Brasileiro, Lash Lifting) ou sobre manutenções e valores antes de agendar.
-Desenvolvemos o *LashMenu*, um catálogo digital interativo feito sob medida para Lash Designers enviar pelo WhatsApp e colocar na Bio do Instagram. Ele organiza seus procedimentos, tabela de preços e orientações pós-procedimento em um só link profissional, acelerando o agendamento de clientes.
-Posso te enviar uma demonstração gratuita que montamos para o seu estúdio dar uma olhada rápida?</t>
+          <t>Oii Tiffany, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
+Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
+          <t>Que ótimo Tiffany! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
           <t>Rua Jdf 216 quadra 31 lote 8, interfone 2 - Dom Fernando II, Goiânia - GO, 74765-250, Brasil</t>
         </is>
       </c>
-      <c r="M32" t="inlineStr">
+      <c r="N32" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Tiffany%20Araujo%20Lash%20Designer&amp;query_place_id=ChIJPyOILwDtXpMRWQI8aKon9xs</t>
         </is>
@@ -2374,18 +2565,24 @@
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr">
         <is>
-          <t>Oii Luana, tudo bem? 👋 Vi o perfil de excelência do seu estúdio no Jardim Vitoria 2 no Google (19 avaliações no Google! ⭐) e achei seu trabalho impecável.
-Percebi que muitas clientes aí em Goiânia ficam em dúvida sobre qual técnica escolher (Fio a Fio, Volume Russo, Brasileiro, Lash Lifting) ou sobre manutenções e valores antes de agendar.
-Desenvolvemos o *LashMenu*, um catálogo digital interativo feito sob medida para Lash Designers enviar pelo WhatsApp e colocar na Bio do Instagram. Ele organiza seus procedimentos, tabela de preços e orientações pós-procedimento em um só link profissional, acelerando o agendamento de clientes.
-Posso te enviar uma demonstração gratuita que montamos para o seu estúdio dar uma olhada rápida?</t>
+          <t>Oii Luana, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
+Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
+          <t>Que ótimo Luana! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
           <t>Av. Sr. do Bonfim - Jardim Vitoria 2, Goiânia - GO, 74865-390, Brasil</t>
         </is>
       </c>
-      <c r="M33" t="inlineStr">
+      <c r="N33" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Luana%20Alves%20-%20EXTENS%C3%83O%20DE%20C%C3%8DLIOS&amp;query_place_id=ChIJTZAvan_7XpMR2Jg80sZtYfE</t>
         </is>
@@ -2428,18 +2625,24 @@
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr">
         <is>
-          <t>Oii Maiza, tudo bem? 👋 Vi o perfil de excelência do seu estúdio no Setor Recanto das Minas Gerais no Google (16 avaliações no Google! ⭐) e achei seu trabalho impecável.
-Percebi que muitas clientes aí em Goiânia ficam em dúvida sobre qual técnica escolher (Fio a Fio, Volume Russo, Brasileiro, Lash Lifting) ou sobre manutenções e valores antes de agendar.
-Desenvolvemos o *LashMenu*, um catálogo digital interativo feito sob medida para Lash Designers enviar pelo WhatsApp e colocar na Bio do Instagram. Ele organiza seus procedimentos, tabela de preços e orientações pós-procedimento em um só link profissional, acelerando o agendamento de clientes.
-Posso te enviar uma demonstração gratuita que montamos para o seu estúdio dar uma olhada rápida?</t>
+          <t>Oii Maiza, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
+Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
+          <t>Que ótimo Maiza! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
           <t>R. SR - 65, 30 - St. Recanto das Minas Gerais, Goiânia - GO, 74785-490, Brasil</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr">
+      <c r="N34" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Maiza%20Gualberto%20-%20Designer&amp;query_place_id=ChIJTbGrc4_tXpMRh9cp08Blirw</t>
         </is>
@@ -2482,18 +2685,24 @@
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr">
         <is>
-          <t>Oii Stúdio, tudo bem? 👋 Vi o perfil de excelência do seu estúdio no Jardim da Luz no Google (12 avaliações no Google! ⭐) e achei seu trabalho impecável.
-Percebi que muitas clientes aí em Goiânia ficam em dúvida sobre qual técnica escolher (Fio a Fio, Volume Russo, Brasileiro, Lash Lifting) ou sobre manutenções e valores antes de agendar.
-Desenvolvemos o *LashMenu*, um catálogo digital interativo feito sob medida para Lash Designers enviar pelo WhatsApp e colocar na Bio do Instagram. Ele organiza seus procedimentos, tabela de preços e orientações pós-procedimento em um só link profissional, acelerando o agendamento de clientes.
-Posso te enviar uma demonstração gratuita que montamos para o seu estúdio dar uma olhada rápida?</t>
+          <t>Oii Stúdio, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
+Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
+          <t>Que ótimo Stúdio! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
           <t>L.20 (Esquina com a - Avenida Leonardo da Vinci, R. Gen. Rondon - Jardim da Luz, Goiânia - GO, 74000-000, Brasil</t>
         </is>
       </c>
-      <c r="M35" t="inlineStr">
+      <c r="N35" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=St%C3%BAdio%20K%C3%A1ssia%20Bianca&amp;query_place_id=ChIJKcBlqBbxXpMRU98OCKiLOG8</t>
         </is>
@@ -2528,18 +2737,24 @@
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr">
         <is>
-          <t>Oii Jéssica, tudo bem? 👋 Vi o perfil de excelência do seu estúdio no Parque das Amendoeiras no Google (23 avaliações no Google! ⭐) e achei seu trabalho impecável.
-Percebi que muitas clientes aí em Goiânia ficam em dúvida sobre qual técnica escolher (Fio a Fio, Volume Russo, Brasileiro, Lash Lifting) ou sobre manutenções e valores antes de agendar.
-Desenvolvemos o *LashMenu*, um catálogo digital interativo feito sob medida para Lash Designers enviar pelo WhatsApp e colocar na Bio do Instagram. Ele organiza seus procedimentos, tabela de preços e orientações pós-procedimento em um só link profissional, acelerando o agendamento de clientes.
-Posso te enviar uma demonstração gratuita que montamos para o seu estúdio dar uma olhada rápida?</t>
+          <t>Oii Jéssica, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
+Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
+          <t>Que ótimo Jéssica! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
           <t>Av. Paulo Alves da Costa, 320 - Parque das Amendoeiras, Goiânia - GO, 74780-500, Brasil</t>
         </is>
       </c>
-      <c r="M36" t="inlineStr">
+      <c r="N36" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Studio%20J%C3%A9ssica%20Oliveira&amp;query_place_id=ChIJtxsg20btXpMR27Z_7BfJEeE</t>
         </is>
@@ -2582,18 +2797,24 @@
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr">
         <is>
-          <t>Oii Carvalho, tudo bem? 👋 Vi o perfil de excelência do seu estúdio em Goiânia no Google (17 avaliações no Google! ⭐) e achei seu trabalho impecável.
-Percebi que muitas clientes aí em Goiânia ficam em dúvida sobre qual técnica escolher (Fio a Fio, Volume Russo, Brasileiro, Lash Lifting) ou sobre manutenções e valores antes de agendar.
-Desenvolvemos o *LashMenu*, um catálogo digital interativo feito sob medida para Lash Designers enviar pelo WhatsApp e colocar na Bio do Instagram. Ele organiza seus procedimentos, tabela de preços e orientações pós-procedimento em um só link profissional, acelerando o agendamento de clientes.
-Posso te enviar uma demonstração gratuita que montamos para o seu estúdio dar uma olhada rápida?</t>
+          <t>Oii Carvalho, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
+Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
+          <t>Que ótimo Carvalho! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
           <t>Av. Aristóteles, Qd 36 - Lt 01 - Goiânia, GO, 74885-030, Brasil</t>
         </is>
       </c>
-      <c r="M37" t="inlineStr">
+      <c r="N37" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Studio%20Carvalho&amp;query_place_id=ChIJRdU9x2XxXpMRzCGYU9op7jo</t>
         </is>
@@ -2636,18 +2857,24 @@
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr">
         <is>
-          <t>Oii Lanna, tudo bem? 👋 Vi o perfil de excelência do seu estúdio no Parque Atheneu no Google ⭐ e achei seu trabalho impecável.
-Percebi que muitas clientes aí em Goiânia ficam em dúvida sobre qual técnica escolher (Fio a Fio, Volume Russo, Brasileiro, Lash Lifting) ou sobre manutenções e valores antes de agendar.
-Desenvolvemos o *LashMenu*, um catálogo digital interativo feito sob medida para Lash Designers enviar pelo WhatsApp e colocar na Bio do Instagram. Ele organiza seus procedimentos, tabela de preços e orientações pós-procedimento em um só link profissional, acelerando o agendamento de clientes.
-Posso te enviar uma demonstração gratuita que montamos para o seu estúdio dar uma olhada rápida?</t>
+          <t>Oii Lanna, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
+Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
+          <t>Que ótimo Lanna! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
           <t>R. Quatro - Parque Atheneu, Goiânia - GO, 74890-710, Brasil</t>
         </is>
       </c>
-      <c r="M38" t="inlineStr">
+      <c r="N38" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Studio%20Lanna%20Lobo&amp;query_place_id=ChIJVyyXJwDlXpMRWTqlnY4xGBI</t>
         </is>
@@ -2690,18 +2917,24 @@
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr">
         <is>
-          <t>Oii Marques, tudo bem? 👋 Vi o perfil de excelência do seu estúdio no Santo Hilario no Google ⭐ e achei seu trabalho impecável.
-Percebi que muitas clientes aí em Goiânia ficam em dúvida sobre qual técnica escolher (Fio a Fio, Volume Russo, Brasileiro, Lash Lifting) ou sobre manutenções e valores antes de agendar.
-Desenvolvemos o *LashMenu*, um catálogo digital interativo feito sob medida para Lash Designers enviar pelo WhatsApp e colocar na Bio do Instagram. Ele organiza seus procedimentos, tabela de preços e orientações pós-procedimento em um só link profissional, acelerando o agendamento de clientes.
-Posso te enviar uma demonstração gratuita que montamos para o seu estúdio dar uma olhada rápida?</t>
+          <t>Oii Marques, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
+Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
+          <t>Que ótimo Marques! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
           <t>Av. Dom Serafim Gomes Jardim, Qd. 45 - Lt.20 - Santo Hilario, Goiânia - GO, 74780-190, Brasil</t>
         </is>
       </c>
-      <c r="M39" t="inlineStr">
+      <c r="N39" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Faby%20Marques%20Lash%20Designer&amp;query_place_id=ChIJb_Gnc9_tXpMRNJOyzmjiiLo</t>
         </is>
@@ -2744,18 +2977,24 @@
       <c r="J40" t="inlineStr"/>
       <c r="K40" t="inlineStr">
         <is>
-          <t>Oii Sara, tudo bem? 👋 Vi o perfil de excelência do seu estúdio no Setor Recanto das Minas Gerais no Google ⭐ e achei seu trabalho impecável.
-Percebi que muitas clientes aí em Goiânia ficam em dúvida sobre qual técnica escolher (Fio a Fio, Volume Russo, Brasileiro, Lash Lifting) ou sobre manutenções e valores antes de agendar.
-Desenvolvemos o *LashMenu*, um catálogo digital interativo feito sob medida para Lash Designers enviar pelo WhatsApp e colocar na Bio do Instagram. Ele organiza seus procedimentos, tabela de preços e orientações pós-procedimento em um só link profissional, acelerando o agendamento de clientes.
-Posso te enviar uma demonstração gratuita que montamos para o seu estúdio dar uma olhada rápida?</t>
+          <t>Oii Sara, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
+Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
+          <t>Que ótimo Sara! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
           <t>R. SR - 65, 63 - Q90, L41 - St. Recanto das Minas Gerais, Goiânia - GO, 74785-330, Brasil</t>
         </is>
       </c>
-      <c r="M40" t="inlineStr">
+      <c r="N40" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Sara%20de%20Paula%20Lash%20Design&amp;query_place_id=ChIJeXQZdhvtXpMRzNvNw6fbKUI</t>
         </is>
@@ -2790,18 +3029,24 @@
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr">
         <is>
-          <t>Oii Ana, tudo bem? 👋 Vi o perfil de excelência do seu estúdio no Vila Pedroso no Google ⭐ e achei seu trabalho impecável.
-Percebi que muitas clientes aí em Goiânia ficam em dúvida sobre qual técnica escolher (Fio a Fio, Volume Russo, Brasileiro, Lash Lifting) ou sobre manutenções e valores antes de agendar.
-Desenvolvemos o *LashMenu*, um catálogo digital interativo feito sob medida para Lash Designers enviar pelo WhatsApp e colocar na Bio do Instagram. Ele organiza seus procedimentos, tabela de preços e orientações pós-procedimento em um só link profissional, acelerando o agendamento de clientes.
-Posso te enviar uma demonstração gratuita que montamos para o seu estúdio dar uma olhada rápida?</t>
+          <t>Oii Ana, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
+Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
+          <t>Que ótimo Ana! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
           <t>R. 2 - Vila Pedroso, Goiânia - GO, 74770-140, Brasil</t>
         </is>
       </c>
-      <c r="M41" t="inlineStr">
+      <c r="N41" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Ana%20Beatriz%20Lash%20Designer&amp;query_place_id=ChIJJRDbBQDvXpMRiKtXEQ_j6_Q</t>
         </is>

</xml_diff>

<commit_message>
feat: adiciona link do Harmonia Rose e 3a mensagem de fechamento com oferta Pix de R
</commit_message>
<xml_diff>
--- a/Prospecção/Leads_LashDesigner_Goiania.xlsx
+++ b/Prospecção/Leads_LashDesigner_Goiania.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N41"/>
+  <dimension ref="A1:O41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -481,20 +481,25 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Abordagem_Inicial_WhatsApp</t>
+          <t>Abordagem_1_Inicial</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Resposta_Se_Responder_SIM</t>
+          <t>Resposta_2_Demonstracao_SIM</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>Fechamento_3_Oferta_Preco_Pix</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>Endereço</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Link_GoogleMaps</t>
         </is>
@@ -553,16 +558,25 @@
       <c r="L2" t="inlineStr">
         <is>
           <t>Que ótimo Edivania! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+👉 https://lashmenu.com/c/harmonia-rose
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
+          <t>Prontinho Edivania! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
           <t>Av. Anhanguera, 5389 - St. Central, Goiânia - GO, 74043-010, Brasil</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Curso%20Extens%C3%A3o%20de%20c%C3%ADlios%20-%20Studio%20Edivania%20Paiva%20Extens%C3%A3o%20de%20c%C3%ADlios%20Goi%C3%A2nia&amp;query_place_id=ChIJNcJRVe7xXpMRegJRirWTQ3Q</t>
         </is>
@@ -621,16 +635,25 @@
       <c r="L3" t="inlineStr">
         <is>
           <t>Que ótimo Layfer! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+👉 https://lashmenu.com/c/harmonia-rose
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
+          <t>Prontinho Layfer! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
           <t>Av. São João esq. c/ Rua Vitoria, Qd. 9, Lt. 11, Alto da Glória Sala 301., 3º Andar - Alto da Glória, Goiânia - GO, 74815-745, Brasil</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Studio%20Layfer%2C%20C%C3%ADlios%2C%20Micropigmenta%C3%A7%C3%A3o%20e%20Est%C3%A9tica%20-%20St.%20Alto%20da%20Gl%C3%B3ria&amp;query_place_id=ChIJzxi2-6PxXpMRk_q1l5AoAD4</t>
         </is>
@@ -685,16 +708,25 @@
       <c r="L4" t="inlineStr">
         <is>
           <t>Que ótimo Larissa! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+👉 https://lashmenu.com/c/harmonia-rose
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
+          <t>Prontinho Larissa! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
           <t>R. T 1-A, 63 - St. Bueno, Goiânia - GO, 74210-330, Brasil</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Studio%20Larissa%20Lobo.%20Especializado%20em%20sobrancelhas%2C%20c%C3%ADlios%20e%20est%C3%A9tica.&amp;query_place_id=ChIJjchOyjzxXpMRxFD2HiV89GI</t>
         </is>
@@ -749,16 +781,25 @@
       <c r="L5" t="inlineStr">
         <is>
           <t>Que ótimo Leticia! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+👉 https://lashmenu.com/c/harmonia-rose
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
+          <t>Prontinho Leticia! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
           <t>Av. T-15, 1380 - St. Bueno, Goiânia - GO, 74230-010, Brasil</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Extens%C3%A3o%20de%20c%C3%ADlios%20Goiania%20-%20Studio%20Leticia%20Santana%20Lash%20Design&amp;query_place_id=ChIJG9x9B23xXpMRznt7moxKXfw</t>
         </is>
@@ -813,16 +854,25 @@
       <c r="L6" t="inlineStr">
         <is>
           <t>Que ótimo Poliana! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+👉 https://lashmenu.com/c/harmonia-rose
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
+          <t>Prontinho Poliana! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
           <t>R. 1137, 225 - QD; 243 LOTE 2 - St. Marista, Goiânia - GO, 74180-160, Brasil</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Extens%C3%A3o%20de%20c%C3%ADlios%20By%20Poliana%20Souza&amp;query_place_id=ChIJl_ZyRl_xXpMRoMv8tRv3jHo</t>
         </is>
@@ -881,16 +931,25 @@
       <c r="L7" t="inlineStr">
         <is>
           <t>Que ótimo Tanielly! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+👉 https://lashmenu.com/c/harmonia-rose
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
+          <t>Prontinho Tanielly! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
           <t>R. São Luís, 364 - Alto da Glória, Goiânia - GO, 74815-755, Brasil</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Tanielly%20Duarte%20Studio%20Beauty&amp;query_place_id=ChIJw-k52L7xXpMRSfLrH3GEy1E</t>
         </is>
@@ -945,16 +1004,25 @@
       <c r="L8" t="inlineStr">
         <is>
           <t>Que ótimo Serena! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+👉 https://lashmenu.com/c/harmonia-rose
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
+          <t>Prontinho Serena! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
           <t>Edifício Trend Office - R. 72, 325 - Sl 1101 - Jardim Goiás, Goiânia - GO, 74805-480, Brasil</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Serena%20Beauty&amp;query_place_id=ChIJ30V_nJLzXpMRZxr4KhUVXi8</t>
         </is>
@@ -1013,16 +1081,25 @@
       <c r="L9" t="inlineStr">
         <is>
           <t>Que ótimo Cinthya! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+👉 https://lashmenu.com/c/harmonia-rose
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
+          <t>Prontinho Cinthya! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
           <t>Comercial das acácias - Alameda Couto Magalhães, 755 - qd S-28 lt 4 sala 201 - St. Bela Vista, Goiânia - GO, 74823-410, Brasil</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
+      <c r="O9" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Studio%20Cinthya%20Montanini%20Goi%C3%A2nia%2C%20Extens%C3%A3o%20de%20C%C3%ADlios%2C%20Micropigmenta%C3%A7%C3%A3o%20de%20Sobrancelha%2C%20Labial%20e%20alongamento%20de%20unha&amp;query_place_id=ChIJGzUau7jxXpMRuco3wD_9oYU</t>
         </is>
@@ -1081,16 +1158,25 @@
       <c r="L10" t="inlineStr">
         <is>
           <t>Que ótimo Design! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+👉 https://lashmenu.com/c/harmonia-rose
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
+          <t>Prontinho Design! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
           <t>Rua 131 Q Area, 342 - St. Sul, Goiânia - GO, 74093-200, Brasil</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
+      <c r="O10" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Design%20de%20Sobrancelhas%20e%20brow%20lamination%20Goi%C3%A2nia%20-%20Milenne%20Beauty%20Organiq&amp;query_place_id=ChIJKSdJ9xXxXpMR2i-K-1q6l5w</t>
         </is>
@@ -1149,16 +1235,25 @@
       <c r="L11" t="inlineStr">
         <is>
           <t>Que ótimo Design! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+👉 https://lashmenu.com/c/harmonia-rose
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
+          <t>Prontinho Design! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
           <t>R. 217, 930 - Setor Leste Universitário, Goiânia - GO, 74603-090, Brasil</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
+      <c r="O11" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Extens%C3%A3o%20de%20C%C3%ADlios%20e%20Design%20de%20Sobrancelhas%20%7C%20Studio%20Brunna%20Lima%20Beauty%20Goi%C3%A2nia&amp;query_place_id=ChIJr9nEaLHzXpMR93NBR10NBeY</t>
         </is>
@@ -1217,16 +1312,25 @@
       <c r="L12" t="inlineStr">
         <is>
           <t>Que ótimo Bella! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+👉 https://lashmenu.com/c/harmonia-rose
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
+          <t>Prontinho Bella! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
           <t>R. Dona Mariquinha, Qd 21 - Lt 26 sala 01 - Setor Negrão de Lima, Goiânia - GO, 74650-130, Brasil</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr">
+      <c r="O12" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Bella%20C%C3%ADlios%20e%20sobrancelhas&amp;query_place_id=ChIJqcYJEjXyXpMRtnQQ3biylr4</t>
         </is>
@@ -1285,16 +1389,25 @@
       <c r="L13" t="inlineStr">
         <is>
           <t>Que ótimo Maria! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+👉 https://lashmenu.com/c/harmonia-rose
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
+          <t>Prontinho Maria! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
           <t>R. 3, lote 8 - unidade 103 - Parque Atheneu, Goiânia - GO, 74893-130, Brasil</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr">
+      <c r="O13" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Studio%20Maria%20Eug%C3%AAnia%20Sobrancelhas&amp;query_place_id=ChIJU43d51L1XpMRs5E5kKLMxX0</t>
         </is>
@@ -1353,16 +1466,25 @@
       <c r="L14" t="inlineStr">
         <is>
           <t>Que ótimo Mariane! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+👉 https://lashmenu.com/c/harmonia-rose
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
+          <t>Prontinho Mariane! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
           <t>R. Quinze, 47 - Und 201 - Parque Atheneu, Goiânia - GO, 74890-230, Brasil</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr">
+      <c r="O14" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Mariane%20Moreno%20Sobrancelhas&amp;query_place_id=ChIJX1H2g17lXpMRgNeUw_-gzZw</t>
         </is>
@@ -1421,16 +1543,25 @@
       <c r="L15" t="inlineStr">
         <is>
           <t>Que ótimo Isabela! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+👉 https://lashmenu.com/c/harmonia-rose
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
+          <t>Prontinho Isabela! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
           <t>Av. 2ª Radial, Qd. 70 - Lt. 06 Sala 2 - Vila Redencao, Goiânia - GO, 74850-040, Brasil</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr">
+      <c r="O15" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Studio%20Isabela%20Souza%20%7C%20C%C3%ADlios%20e%20Sobrancelhas%20em%20Goi%C3%A2nia&amp;query_place_id=ChIJ6_FUKYnxXpMRZl7o8vNiDJE</t>
         </is>
@@ -1489,16 +1620,25 @@
       <c r="L16" t="inlineStr">
         <is>
           <t>Que ótimo Déborah! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+👉 https://lashmenu.com/c/harmonia-rose
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
+          <t>Prontinho Déborah! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
           <t>Sobrancelha Natural, Cílios, Design, Henna Cílios em - R. C-252, N° 1141 - QD 604, LT 11 - Nova Suiça, Goiânia - GO, 74280-160, Brasil</t>
         </is>
       </c>
-      <c r="N16" t="inlineStr">
+      <c r="O16" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=D%C3%A9borah%20Alvarenga%20Beauty%20-%20C%C3%ADlios%20Goi%C3%A2nia%20%2F%20Sobrancelha%20Natural%20%2F%20C%C3%ADlios&amp;query_place_id=ChIJl9chJ-nxXpMRqLdSKfOsPEI</t>
         </is>
@@ -1557,16 +1697,25 @@
       <c r="L17" t="inlineStr">
         <is>
           <t>Que ótimo Yara! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+👉 https://lashmenu.com/c/harmonia-rose
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
+          <t>Prontinho Yara! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
           <t>R. Poe. Joaquim Bonifácio - Goiânia, GO, 74770-410, Brasil</t>
         </is>
       </c>
-      <c r="N17" t="inlineStr">
+      <c r="O17" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Yara%20Ferreira%20Lash%20Designer%20-%20Extens%C3%A3o%20de%20C%C3%ADlios&amp;query_place_id=ChIJyxTL8p7vXpMR1pVLBLcrUEg</t>
         </is>
@@ -1621,16 +1770,25 @@
       <c r="L18" t="inlineStr">
         <is>
           <t>Que ótimo Kathellem! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+👉 https://lashmenu.com/c/harmonia-rose
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
+          <t>Prontinho Kathellem! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
           <t>R. 233, 1483 - Qd 78 Lt 12 - Setor Leste Universitário, Goiânia - GO, 74605-120, Brasil</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr">
+      <c r="O18" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Studio%20Kathellem%20lima%20-%20Lash%20Designer%20(Extens%C3%A3o%20de%20c%C3%ADlios)-%20Designer%20de%20sobrancelha%20-%20maquiagem-Depila%C3%A7%C3%A3o&amp;query_place_id=ChIJlQQGMQzxXpMRzMyTFfdm_pU</t>
         </is>
@@ -1685,16 +1843,25 @@
       <c r="L19" t="inlineStr">
         <is>
           <t>Que ótimo Lollys! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+👉 https://lashmenu.com/c/harmonia-rose
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
+          <t>Prontinho Lollys! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
           <t>Av. C-255, 271 - Nova Suiça, Goiânia - GO, 74280-010, Brasil</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr">
+      <c r="O19" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Studio%20Lollys%20Cilios&amp;query_place_id=ChIJGye0ibH2XpMRF8fxewDzYv4</t>
         </is>
@@ -1745,16 +1912,25 @@
       <c r="L20" t="inlineStr">
         <is>
           <t>Que ótimo Ariana! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+👉 https://lashmenu.com/c/harmonia-rose
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
+          <t>Prontinho Ariana! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
           <t>R. 209-A, 1405 - Leste Vila Nova, Goiânia - GO, 74645-210, Brasil</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr">
+      <c r="O20" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=EXTENS%C3%83O%20DE%20C%C3%8DLIOS%20GOI%C3%82NIA-%20ARIANA&amp;query_place_id=ChIJOU-jj6jzXpMROoQLtO7YqUw</t>
         </is>
@@ -1805,16 +1981,25 @@
       <c r="L21" t="inlineStr">
         <is>
           <t>Que ótimo Design! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+👉 https://lashmenu.com/c/harmonia-rose
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
+          <t>Prontinho Design! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
           <t>Qd F37 28, R. 88-D, 286 - St. Sul, Goiânia - GO, 74085-115, Brasil</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr">
+      <c r="O21" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Sobrancelhas%20Design&amp;query_place_id=ChIJv6BTMnPxXpMRSTgLft6uVY4</t>
         </is>
@@ -1873,16 +2058,25 @@
       <c r="L22" t="inlineStr">
         <is>
           <t>Que ótimo Elaíne! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+👉 https://lashmenu.com/c/harmonia-rose
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
+          <t>Prontinho Elaíne! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
           <t>Av. Francisco Ludovíco de Almeida, qd35 lote17 - Parque das Amendoeiras, Goiânia - GO, 74780-440, Brasil</t>
         </is>
       </c>
-      <c r="N22" t="inlineStr">
+      <c r="O22" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Ela%C3%ADne%20Nascimento%20Lashdesigner%20-%20Extens%C3%A3o%20de%20c%C3%ADlios%20e%20Designer%20de%20Sobrancelha%20em%20Goi%C3%A2nia&amp;query_place_id=ChIJB0t6XAztXpMRfyugbg31EHw</t>
         </is>
@@ -1937,16 +2131,25 @@
       <c r="L23" t="inlineStr">
         <is>
           <t>Que ótimo Cílios! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+👉 https://lashmenu.com/c/harmonia-rose
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
+          <t>Prontinho Cílios! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
           <t>R. João Luís, qd 07 - LT 07 - Bairro Santa Rita, Goiânia - GO, 74370-580, Brasil</t>
         </is>
       </c>
-      <c r="N23" t="inlineStr">
+      <c r="O23" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Extens%C3%A3o%20de%20C%C3%ADlios%20-%20Studio%20de%20C%C3%ADlios%20Nayara&amp;query_place_id=ChIJG8ux-Ov3XpMRWf58BW9LZ5c</t>
         </is>
@@ -2005,16 +2208,25 @@
       <c r="L24" t="inlineStr">
         <is>
           <t>Que ótimo Joana! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+👉 https://lashmenu.com/c/harmonia-rose
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
+          <t>Prontinho Joana! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
           <t>R. 9, qd 09 lt 02 casa 1 - Residencial Paulo estrela, Goiânia - GO, 74786-444, Brasil</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr">
+      <c r="O24" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Joana%20Paiva%20studio&amp;query_place_id=ChIJJ3J5bgntXpMRud_xJ4tempE</t>
         </is>
@@ -2069,16 +2281,25 @@
       <c r="L25" t="inlineStr">
         <is>
           <t>Que ótimo Cílios! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+👉 https://lashmenu.com/c/harmonia-rose
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
+          <t>Prontinho Cílios! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
           <t>R. Gen. Braz Arantes, 129 - qd09 lt11 - Crimeia Leste, Goiânia - GO, 74660-210, Brasil</t>
         </is>
       </c>
-      <c r="N25" t="inlineStr">
+      <c r="O25" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=C%C3%ADlios%20Showroom&amp;query_place_id=ChIJu0BGTGvzXpMRocxq8JKc-Sw</t>
         </is>
@@ -2133,16 +2354,25 @@
       <c r="L26" t="inlineStr">
         <is>
           <t>Que ótimo Katyane! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+👉 https://lashmenu.com/c/harmonia-rose
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
+          <t>Prontinho Katyane! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
           <t>Rua 2031, R. 1 Unidade 203 - Parque Atheneu, Goiânia - GO, 74890-700, Brasil</t>
         </is>
       </c>
-      <c r="N26" t="inlineStr">
+      <c r="O26" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Studio%20Katyane%20Mendes&amp;query_place_id=ChIJDWwGdzblXpMRd3FPc_MqTIE</t>
         </is>
@@ -2193,16 +2423,25 @@
       <c r="L27" t="inlineStr">
         <is>
           <t>Que ótimo Vidal! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+👉 https://lashmenu.com/c/harmonia-rose
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
+          <t>Prontinho Vidal! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
           <t>Rua 101 unid101, lote 2, Goiânia - GO, 74893-530, Brasil</t>
         </is>
       </c>
-      <c r="N27" t="inlineStr">
+      <c r="O27" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Studio%20Vidal%20Priscila&amp;query_place_id=ChIJy5B_VJv7XpMRvSe-I9ZXO6M</t>
         </is>
@@ -2253,16 +2492,25 @@
       <c r="L28" t="inlineStr">
         <is>
           <t>Que ótimo Crys! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+👉 https://lashmenu.com/c/harmonia-rose
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
+          <t>Prontinho Crys! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
           <t>Av. F, quadra A - lote 04 - Setor - Água Branca, Goiânia - GO, 74730-320, Brasil</t>
         </is>
       </c>
-      <c r="N28" t="inlineStr">
+      <c r="O28" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Crys%20Lohany%20Lashes&amp;query_place_id=ChIJE3PPbB7xXpMR8fpw2IcHaEo</t>
         </is>
@@ -2313,16 +2561,25 @@
       <c r="L29" t="inlineStr">
         <is>
           <t>Que ótimo Aliany! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+👉 https://lashmenu.com/c/harmonia-rose
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
+          <t>Prontinho Aliany! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
           <t>Av. Bela Vista, qd i lt1 - Jardim Bela Vista, Goiânia - GO, 74863-050, Brasil</t>
         </is>
       </c>
-      <c r="N29" t="inlineStr">
+      <c r="O29" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Studio%20Aliany%20Mendes%20-%20Nail%20Designer&amp;query_place_id=ChIJkUJBKqrxXpMR6xxIrqyhBBg</t>
         </is>
@@ -2377,16 +2634,25 @@
       <c r="L30" t="inlineStr">
         <is>
           <t>Que ótimo D'isanto! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+👉 https://lashmenu.com/c/harmonia-rose
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
+          <t>Prontinho D'isanto! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
           <t>R. Caraíba - Jardim Mariliza, Goiânia - GO, 74885-090, Brasil</t>
         </is>
       </c>
-      <c r="N30" t="inlineStr">
+      <c r="O30" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=D'Isanto%20Brows%20%7C%20Design%20de%20Sobrancelhas%20%7C%20Brow%20Lamination%20%7C%20Lash%20Lifting&amp;query_place_id=ChIJURiAgEv7XpMRzE1r8meSquY</t>
         </is>
@@ -2445,16 +2711,25 @@
       <c r="L31" t="inlineStr">
         <is>
           <t>Que ótimo Ynnaê! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+👉 https://lashmenu.com/c/harmonia-rose
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
+          <t>Prontinho Ynnaê! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
           <t>R. JDA Dez, Quadra 07 lote 14 sala 01 - Jardim das Aroeiras, Goiânia - GO, 74770-550, Brasil</t>
         </is>
       </c>
-      <c r="N31" t="inlineStr">
+      <c r="O31" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Ynna%C3%AA%20Uch%C3%B4a%20Lash%20Design%20Micropigmentadora&amp;query_place_id=ChIJiTtbqZfvXpMRIO3w6gfFvF8</t>
         </is>
@@ -2513,16 +2788,25 @@
       <c r="L32" t="inlineStr">
         <is>
           <t>Que ótimo Tiffany! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+👉 https://lashmenu.com/c/harmonia-rose
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
+          <t>Prontinho Tiffany! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
           <t>Rua Jdf 216 quadra 31 lote 8, interfone 2 - Dom Fernando II, Goiânia - GO, 74765-250, Brasil</t>
         </is>
       </c>
-      <c r="N32" t="inlineStr">
+      <c r="O32" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Tiffany%20Araujo%20Lash%20Designer&amp;query_place_id=ChIJPyOILwDtXpMRWQI8aKon9xs</t>
         </is>
@@ -2573,16 +2857,25 @@
       <c r="L33" t="inlineStr">
         <is>
           <t>Que ótimo Luana! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+👉 https://lashmenu.com/c/harmonia-rose
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
+          <t>Prontinho Luana! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
           <t>Av. Sr. do Bonfim - Jardim Vitoria 2, Goiânia - GO, 74865-390, Brasil</t>
         </is>
       </c>
-      <c r="N33" t="inlineStr">
+      <c r="O33" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Luana%20Alves%20-%20EXTENS%C3%83O%20DE%20C%C3%8DLIOS&amp;query_place_id=ChIJTZAvan_7XpMR2Jg80sZtYfE</t>
         </is>
@@ -2633,16 +2926,25 @@
       <c r="L34" t="inlineStr">
         <is>
           <t>Que ótimo Maiza! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+👉 https://lashmenu.com/c/harmonia-rose
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
+          <t>Prontinho Maiza! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
           <t>R. SR - 65, 30 - St. Recanto das Minas Gerais, Goiânia - GO, 74785-490, Brasil</t>
         </is>
       </c>
-      <c r="N34" t="inlineStr">
+      <c r="O34" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Maiza%20Gualberto%20-%20Designer&amp;query_place_id=ChIJTbGrc4_tXpMRh9cp08Blirw</t>
         </is>
@@ -2693,16 +2995,25 @@
       <c r="L35" t="inlineStr">
         <is>
           <t>Que ótimo Stúdio! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+👉 https://lashmenu.com/c/harmonia-rose
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
+          <t>Prontinho Stúdio! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
           <t>L.20 (Esquina com a - Avenida Leonardo da Vinci, R. Gen. Rondon - Jardim da Luz, Goiânia - GO, 74000-000, Brasil</t>
         </is>
       </c>
-      <c r="N35" t="inlineStr">
+      <c r="O35" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=St%C3%BAdio%20K%C3%A1ssia%20Bianca&amp;query_place_id=ChIJKcBlqBbxXpMRU98OCKiLOG8</t>
         </is>
@@ -2745,16 +3056,25 @@
       <c r="L36" t="inlineStr">
         <is>
           <t>Que ótimo Jéssica! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+👉 https://lashmenu.com/c/harmonia-rose
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
+          <t>Prontinho Jéssica! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
           <t>Av. Paulo Alves da Costa, 320 - Parque das Amendoeiras, Goiânia - GO, 74780-500, Brasil</t>
         </is>
       </c>
-      <c r="N36" t="inlineStr">
+      <c r="O36" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Studio%20J%C3%A9ssica%20Oliveira&amp;query_place_id=ChIJtxsg20btXpMR27Z_7BfJEeE</t>
         </is>
@@ -2805,16 +3125,25 @@
       <c r="L37" t="inlineStr">
         <is>
           <t>Que ótimo Carvalho! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+👉 https://lashmenu.com/c/harmonia-rose
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
+          <t>Prontinho Carvalho! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
           <t>Av. Aristóteles, Qd 36 - Lt 01 - Goiânia, GO, 74885-030, Brasil</t>
         </is>
       </c>
-      <c r="N37" t="inlineStr">
+      <c r="O37" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Studio%20Carvalho&amp;query_place_id=ChIJRdU9x2XxXpMRzCGYU9op7jo</t>
         </is>
@@ -2865,16 +3194,25 @@
       <c r="L38" t="inlineStr">
         <is>
           <t>Que ótimo Lanna! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+👉 https://lashmenu.com/c/harmonia-rose
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
+          <t>Prontinho Lanna! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
           <t>R. Quatro - Parque Atheneu, Goiânia - GO, 74890-710, Brasil</t>
         </is>
       </c>
-      <c r="N38" t="inlineStr">
+      <c r="O38" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Studio%20Lanna%20Lobo&amp;query_place_id=ChIJVyyXJwDlXpMRWTqlnY4xGBI</t>
         </is>
@@ -2925,16 +3263,25 @@
       <c r="L39" t="inlineStr">
         <is>
           <t>Que ótimo Marques! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+👉 https://lashmenu.com/c/harmonia-rose
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
+          <t>Prontinho Marques! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
           <t>Av. Dom Serafim Gomes Jardim, Qd. 45 - Lt.20 - Santo Hilario, Goiânia - GO, 74780-190, Brasil</t>
         </is>
       </c>
-      <c r="N39" t="inlineStr">
+      <c r="O39" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Faby%20Marques%20Lash%20Designer&amp;query_place_id=ChIJb_Gnc9_tXpMRNJOyzmjiiLo</t>
         </is>
@@ -2985,16 +3332,25 @@
       <c r="L40" t="inlineStr">
         <is>
           <t>Que ótimo Sara! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+👉 https://lashmenu.com/c/harmonia-rose
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
+          <t>Prontinho Sara! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
           <t>R. SR - 65, 63 - Q90, L41 - St. Recanto das Minas Gerais, Goiânia - GO, 74785-330, Brasil</t>
         </is>
       </c>
-      <c r="N40" t="inlineStr">
+      <c r="O40" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Sara%20de%20Paula%20Lash%20Design&amp;query_place_id=ChIJeXQZdhvtXpMRzNvNw6fbKUI</t>
         </is>
@@ -3037,16 +3393,25 @@
       <c r="L41" t="inlineStr">
         <is>
           <t>Que ótimo Ana! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 [INSERIR LINK DO DEMO AQUI - Ex: modelo Harmonia Rose]
+👉 https://lashmenu.com/c/harmonia-rose
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
         <is>
+          <t>Prontinho Ana! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
           <t>R. 2 - Vila Pedroso, Goiânia - GO, 74770-140, Brasil</t>
         </is>
       </c>
-      <c r="N41" t="inlineStr">
+      <c r="O41" t="inlineStr">
         <is>
           <t>https://www.google.com/maps/search/?api=1&amp;query=Ana%20Beatriz%20Lash%20Designer&amp;query_place_id=ChIJJRDbBQDvXpMRiKtXEQ_j6_Q</t>
         </is>

</xml_diff>

<commit_message>
style: adiciona emojis e quebra de linha nas mensagens de abordagem
</commit_message>
<xml_diff>
--- a/Prospecção/Leads_LashDesigner_Goiania.xlsx
+++ b/Prospecção/Leads_LashDesigner_Goiania.xlsx
@@ -550,25 +550,26 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Oii Edivania, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
-Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
-Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
+          <t>Oii Edivania, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
+Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
+Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Que ótimo Edivania! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+          <t>Que ótimo Edivania! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 https://lashmenu.com/c/harmonia-rose ✨
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Prontinho Edivania! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
-👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
-A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
-Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
-Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+          <t>Prontinho Edivania! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo? 🚀💕</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -627,25 +628,26 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Oii Layfer, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
-Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
-Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
+          <t>Oii Layfer, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
+Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
+Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Que ótimo Layfer! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+          <t>Que ótimo Layfer! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 https://lashmenu.com/c/harmonia-rose ✨
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Prontinho Layfer! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
-👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
-A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
-Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
-Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+          <t>Prontinho Layfer! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo? 🚀💕</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -700,25 +702,26 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Oii Larissa, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
-Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
-Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
+          <t>Oii Larissa, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
+Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
+Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Que ótimo Larissa! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+          <t>Que ótimo Larissa! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 https://lashmenu.com/c/harmonia-rose ✨
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Prontinho Larissa! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
-👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
-A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
-Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
-Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+          <t>Prontinho Larissa! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo? 🚀💕</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -773,25 +776,26 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Oii Leticia, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
-Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
-Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
+          <t>Oii Leticia, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
+Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
+Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Que ótimo Leticia! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+          <t>Que ótimo Leticia! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 https://lashmenu.com/c/harmonia-rose ✨
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Prontinho Leticia! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
-👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
-A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
-Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
-Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+          <t>Prontinho Leticia! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo? 🚀💕</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -846,25 +850,26 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Oii Poliana, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
-Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
-Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
+          <t>Oii Poliana, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
+Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
+Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Que ótimo Poliana! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+          <t>Que ótimo Poliana! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 https://lashmenu.com/c/harmonia-rose ✨
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Prontinho Poliana! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
-👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
-A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
-Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
-Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+          <t>Prontinho Poliana! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo? 🚀💕</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -923,25 +928,26 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Oii Tanielly, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
-Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
-Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
+          <t>Oii Tanielly, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
+Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
+Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Que ótimo Tanielly! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+          <t>Que ótimo Tanielly! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 https://lashmenu.com/c/harmonia-rose ✨
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Prontinho Tanielly! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
-👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
-A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
-Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
-Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+          <t>Prontinho Tanielly! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo? 🚀💕</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -996,25 +1002,26 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Oii Serena, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
-Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
-Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
+          <t>Oii Serena, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
+Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
+Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Que ótimo Serena! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+          <t>Que ótimo Serena! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 https://lashmenu.com/c/harmonia-rose ✨
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Prontinho Serena! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
-👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
-A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
-Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
-Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+          <t>Prontinho Serena! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo? 🚀💕</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1073,25 +1080,26 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Oii Cinthya, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
-Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
-Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
+          <t>Oii Cinthya, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
+Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
+Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Que ótimo Cinthya! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+          <t>Que ótimo Cinthya! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 https://lashmenu.com/c/harmonia-rose ✨
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Prontinho Cinthya! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
-👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
-A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
-Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
-Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+          <t>Prontinho Cinthya! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo? 🚀💕</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1150,25 +1158,26 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Oii Design, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
-Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
-Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
+          <t>Oii Design, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
+Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
+Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Que ótimo Design! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+          <t>Que ótimo Design! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 https://lashmenu.com/c/harmonia-rose ✨
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Prontinho Design! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
-👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
-A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
-Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
-Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+          <t>Prontinho Design! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo? 🚀💕</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1227,25 +1236,26 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Oii Design, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
-Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
-Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
+          <t>Oii Design, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
+Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
+Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Que ótimo Design! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+          <t>Que ótimo Design! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 https://lashmenu.com/c/harmonia-rose ✨
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Prontinho Design! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
-👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
-A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
-Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
-Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+          <t>Prontinho Design! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo? 🚀💕</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1304,25 +1314,26 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Oii Bella, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
-Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
-Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
+          <t>Oii Bella, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
+Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
+Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Que ótimo Bella! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+          <t>Que ótimo Bella! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 https://lashmenu.com/c/harmonia-rose ✨
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Prontinho Bella! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
-👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
-A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
-Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
-Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+          <t>Prontinho Bella! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo? 🚀💕</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1381,25 +1392,26 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Oii Maria, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
-Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
-Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
+          <t>Oii Maria, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
+Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
+Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>Que ótimo Maria! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+          <t>Que ótimo Maria! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 https://lashmenu.com/c/harmonia-rose ✨
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Prontinho Maria! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
-👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
-A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
-Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
-Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+          <t>Prontinho Maria! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo? 🚀💕</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1458,25 +1470,26 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Oii Mariane, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
-Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
-Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
+          <t>Oii Mariane, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
+Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
+Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Que ótimo Mariane! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+          <t>Que ótimo Mariane! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 https://lashmenu.com/c/harmonia-rose ✨
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Prontinho Mariane! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
-👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
-A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
-Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
-Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+          <t>Prontinho Mariane! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo? 🚀💕</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1535,25 +1548,26 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Oii Isabela, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
-Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
-Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
+          <t>Oii Isabela, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
+Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
+Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Que ótimo Isabela! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+          <t>Que ótimo Isabela! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 https://lashmenu.com/c/harmonia-rose ✨
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Prontinho Isabela! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
-👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
-A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
-Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
-Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+          <t>Prontinho Isabela! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo? 🚀💕</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1612,25 +1626,26 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Oii Déborah, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
-Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
-Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
+          <t>Oii Déborah, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
+Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
+Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Que ótimo Déborah! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+          <t>Que ótimo Déborah! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 https://lashmenu.com/c/harmonia-rose ✨
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Prontinho Déborah! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
-👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
-A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
-Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
-Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+          <t>Prontinho Déborah! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo? 🚀💕</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -1689,25 +1704,26 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Oii Yara, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
-Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
-Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
+          <t>Oii Yara, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
+Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
+Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Que ótimo Yara! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+          <t>Que ótimo Yara! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 https://lashmenu.com/c/harmonia-rose ✨
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>Prontinho Yara! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
-👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
-A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
-Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
-Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+          <t>Prontinho Yara! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo? 🚀💕</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -1762,25 +1778,26 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Oii Kathellem, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
-Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
-Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
+          <t>Oii Kathellem, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
+Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
+Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Que ótimo Kathellem! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+          <t>Que ótimo Kathellem! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 https://lashmenu.com/c/harmonia-rose ✨
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>Prontinho Kathellem! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
-👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
-A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
-Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
-Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+          <t>Prontinho Kathellem! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo? 🚀💕</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -1835,25 +1852,26 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Oii Lollys, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
-Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
-Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
+          <t>Oii Lollys, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
+Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
+Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Que ótimo Lollys! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+          <t>Que ótimo Lollys! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 https://lashmenu.com/c/harmonia-rose ✨
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>Prontinho Lollys! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
-👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
-A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
-Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
-Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+          <t>Prontinho Lollys! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo? 🚀💕</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -1904,25 +1922,26 @@
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Oii Ariana, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
-Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
-Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
+          <t>Oii Ariana, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
+Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
+Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Que ótimo Ariana! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+          <t>Que ótimo Ariana! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 https://lashmenu.com/c/harmonia-rose ✨
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>Prontinho Ariana! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
-👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
-A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
-Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
-Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+          <t>Prontinho Ariana! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo? 🚀💕</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -1973,25 +1992,26 @@
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Oii Design, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
-Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
-Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
+          <t>Oii Design, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
+Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
+Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Que ótimo Design! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+          <t>Que ótimo Design! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 https://lashmenu.com/c/harmonia-rose ✨
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>Prontinho Design! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
-👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
-A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
-Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
-Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+          <t>Prontinho Design! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo? 🚀💕</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -2050,25 +2070,26 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Oii Elaíne, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
-Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
-Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
+          <t>Oii Elaíne, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
+Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
+Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Que ótimo Elaíne! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+          <t>Que ótimo Elaíne! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 https://lashmenu.com/c/harmonia-rose ✨
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>Prontinho Elaíne! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
-👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
-A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
-Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
-Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+          <t>Prontinho Elaíne! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo? 🚀💕</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -2123,25 +2144,26 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Oii Cílios, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
-Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
-Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
+          <t>Oii Cílios, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
+Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
+Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Que ótimo Cílios! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+          <t>Que ótimo Cílios! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 https://lashmenu.com/c/harmonia-rose ✨
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>Prontinho Cílios! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
-👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
-A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
-Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
-Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+          <t>Prontinho Cílios! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo? 🚀💕</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -2200,25 +2222,26 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Oii Joana, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
-Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
-Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
+          <t>Oii Joana, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
+Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
+Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Que ótimo Joana! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+          <t>Que ótimo Joana! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 https://lashmenu.com/c/harmonia-rose ✨
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>Prontinho Joana! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
-👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
-A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
-Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
-Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+          <t>Prontinho Joana! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo? 🚀💕</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -2273,25 +2296,26 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Oii Cílios, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
-Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
-Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
+          <t>Oii Cílios, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
+Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
+Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>Que ótimo Cílios! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+          <t>Que ótimo Cílios! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 https://lashmenu.com/c/harmonia-rose ✨
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>Prontinho Cílios! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
-👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
-A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
-Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
-Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+          <t>Prontinho Cílios! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo? 🚀💕</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -2346,25 +2370,26 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Oii Katyane, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
-Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
-Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
+          <t>Oii Katyane, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
+Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
+Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Que ótimo Katyane! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+          <t>Que ótimo Katyane! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 https://lashmenu.com/c/harmonia-rose ✨
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>Prontinho Katyane! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
-👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
-A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
-Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
-Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+          <t>Prontinho Katyane! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo? 🚀💕</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -2415,25 +2440,26 @@
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Oii Vidal, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
-Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
-Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
+          <t>Oii Vidal, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
+Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
+Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>Que ótimo Vidal! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+          <t>Que ótimo Vidal! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 https://lashmenu.com/c/harmonia-rose ✨
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>Prontinho Vidal! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
-👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
-A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
-Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
-Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+          <t>Prontinho Vidal! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo? 🚀💕</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -2484,25 +2510,26 @@
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr">
         <is>
-          <t>Oii Crys, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
-Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
-Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
+          <t>Oii Crys, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
+Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
+Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>Que ótimo Crys! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+          <t>Que ótimo Crys! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 https://lashmenu.com/c/harmonia-rose ✨
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>Prontinho Crys! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
-👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
-A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
-Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
-Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+          <t>Prontinho Crys! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo? 🚀💕</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -2553,25 +2580,26 @@
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Oii Aliany, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
-Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
-Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
+          <t>Oii Aliany, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
+Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
+Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>Que ótimo Aliany! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+          <t>Que ótimo Aliany! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 https://lashmenu.com/c/harmonia-rose ✨
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>Prontinho Aliany! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
-👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
-A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
-Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
-Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+          <t>Prontinho Aliany! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo? 🚀💕</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2626,25 +2654,26 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Oii D'isanto, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
-Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
-Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
+          <t>Oii D'isanto, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
+Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
+Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>Que ótimo D'isanto! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+          <t>Que ótimo D'isanto! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 https://lashmenu.com/c/harmonia-rose ✨
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>Prontinho D'isanto! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
-👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
-A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
-Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
-Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+          <t>Prontinho D'isanto! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo? 🚀💕</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -2703,25 +2732,26 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Oii Ynnaê, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
-Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
-Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
+          <t>Oii Ynnaê, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
+Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
+Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>Que ótimo Ynnaê! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+          <t>Que ótimo Ynnaê! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 https://lashmenu.com/c/harmonia-rose ✨
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>Prontinho Ynnaê! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
-👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
-A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
-Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
-Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+          <t>Prontinho Ynnaê! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo? 🚀💕</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -2780,25 +2810,26 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>Oii Tiffany, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
-Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
-Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
+          <t>Oii Tiffany, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
+Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
+Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>Que ótimo Tiffany! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+          <t>Que ótimo Tiffany! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 https://lashmenu.com/c/harmonia-rose ✨
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>Prontinho Tiffany! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
-👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
-A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
-Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
-Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+          <t>Prontinho Tiffany! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo? 🚀💕</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -2849,25 +2880,26 @@
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr">
         <is>
-          <t>Oii Luana, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
-Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
-Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
+          <t>Oii Luana, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
+Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
+Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>Que ótimo Luana! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+          <t>Que ótimo Luana! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 https://lashmenu.com/c/harmonia-rose ✨
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>Prontinho Luana! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
-👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
-A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
-Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
-Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+          <t>Prontinho Luana! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo? 🚀💕</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -2918,25 +2950,26 @@
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr">
         <is>
-          <t>Oii Maiza, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
-Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
-Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
+          <t>Oii Maiza, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
+Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
+Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>Que ótimo Maiza! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+          <t>Que ótimo Maiza! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 https://lashmenu.com/c/harmonia-rose ✨
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>Prontinho Maiza! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
-👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
-A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
-Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
-Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+          <t>Prontinho Maiza! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo? 🚀💕</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -2987,25 +3020,26 @@
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr">
         <is>
-          <t>Oii Stúdio, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
-Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
-Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
+          <t>Oii Stúdio, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
+Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
+Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>Que ótimo Stúdio! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+          <t>Que ótimo Stúdio! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 https://lashmenu.com/c/harmonia-rose ✨
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>Prontinho Stúdio! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
-👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
-A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
-Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
-Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+          <t>Prontinho Stúdio! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo? 🚀💕</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
@@ -3048,25 +3082,26 @@
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr">
         <is>
-          <t>Oii Jéssica, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
-Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
-Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
+          <t>Oii Jéssica, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
+Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
+Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>Que ótimo Jéssica! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+          <t>Que ótimo Jéssica! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 https://lashmenu.com/c/harmonia-rose ✨
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>Prontinho Jéssica! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
-👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
-A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
-Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
-Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+          <t>Prontinho Jéssica! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo? 🚀💕</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
@@ -3117,25 +3152,26 @@
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr">
         <is>
-          <t>Oii Carvalho, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
-Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
-Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
+          <t>Oii Carvalho, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
+Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
+Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>Que ótimo Carvalho! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+          <t>Que ótimo Carvalho! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 https://lashmenu.com/c/harmonia-rose ✨
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>Prontinho Carvalho! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
-👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
-A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
-Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
-Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+          <t>Prontinho Carvalho! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo? 🚀💕</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -3186,25 +3222,26 @@
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr">
         <is>
-          <t>Oii Lanna, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
-Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
-Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
+          <t>Oii Lanna, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
+Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
+Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>Que ótimo Lanna! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+          <t>Que ótimo Lanna! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 https://lashmenu.com/c/harmonia-rose ✨
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>Prontinho Lanna! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
-👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
-A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
-Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
-Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+          <t>Prontinho Lanna! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo? 🚀💕</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -3255,25 +3292,26 @@
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr">
         <is>
-          <t>Oii Marques, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
-Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
-Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
+          <t>Oii Marques, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
+Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
+Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>Que ótimo Marques! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+          <t>Que ótimo Marques! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 https://lashmenu.com/c/harmonia-rose ✨
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>Prontinho Marques! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
-👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
-A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
-Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
-Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+          <t>Prontinho Marques! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo? 🚀💕</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -3324,25 +3362,26 @@
       <c r="J40" t="inlineStr"/>
       <c r="K40" t="inlineStr">
         <is>
-          <t>Oii Sara, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
-Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
-Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
+          <t>Oii Sara, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
+Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
+Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>Que ótimo Sara! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+          <t>Que ótimo Sara! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 https://lashmenu.com/c/harmonia-rose ✨
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>Prontinho Sara! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
-👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
-A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
-Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
-Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+          <t>Prontinho Sara! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo? 🚀💕</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -3385,25 +3424,26 @@
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr">
         <is>
-          <t>Oii Ana, tudo bem? 👋 Vi o seu perfil no Google e achei os seus trabalhos de cílios incríveis!
-Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os agendamentos.
-Posso te mandar um modelo de demonstração para você ver como fica na prática?</t>
+          <t>Oii Ana, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
+Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
+Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>Que ótimo Ana! 💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática!</t>
+          <t>Que ótimo Ana! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+👉 https://lashmenu.com/c/harmonia-rose ✨
+Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>Prontinho Ana! 🌸 Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
-👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA]
-A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
-Mas como estamos falando diretamente por aqui no WhatsApp, conseguimos uma condição especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único)*!
-Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo?</t>
+          <t>Prontinho Ana! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
+A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
+Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
+Quer que eu já te envie a chave Pix para liberarmos o seu link definitivo hoje mesmo? 🚀💕</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">

</xml_diff>

<commit_message>
fix: corrige e valida 100% dos nomes das Lash Designers para todas as 40 abordagens
</commit_message>
<xml_diff>
--- a/Prospecção/Leads_LashDesigner_Goiania.xlsx
+++ b/Prospecção/Leads_LashDesigner_Goiania.xlsx
@@ -1158,7 +1158,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Oii Design, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+          <t>Oii Milenne, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
 Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
 Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
 Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
@@ -1166,14 +1166,14 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Que ótimo Design! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+          <t>Que ótimo Milenne! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
 👉 https://lashmenu.com/c/harmonia-rose ✨
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Prontinho Design! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+          <t>Prontinho Milenne! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
 👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
 A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
 Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
@@ -1236,7 +1236,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Oii Design, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+          <t>Oii Brunna, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
 Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
 Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
 Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
@@ -1244,14 +1244,14 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Que ótimo Design! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+          <t>Que ótimo Brunna! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
 👉 https://lashmenu.com/c/harmonia-rose ✨
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Prontinho Design! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+          <t>Prontinho Brunna! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
 👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
 A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
 Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
@@ -1392,7 +1392,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Oii Maria, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+          <t>Oii Maria Eugênia, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
 Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
 Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
 Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
@@ -1400,14 +1400,14 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>Que ótimo Maria! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+          <t>Que ótimo Maria Eugênia! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
 👉 https://lashmenu.com/c/harmonia-rose ✨
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Prontinho Maria! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+          <t>Prontinho Maria Eugênia! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
 👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
 A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
 Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
@@ -1992,7 +1992,7 @@
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Oii Design, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+          <t>Oii, tudo bem?, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
 Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
 Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
 Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
@@ -2000,14 +2000,14 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Que ótimo Design! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+          <t>Que ótimo! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
 👉 https://lashmenu.com/c/harmonia-rose ✨
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>Prontinho Design! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+          <t>Prontinho! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
 👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
 A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
 Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
@@ -2144,7 +2144,7 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Oii Cílios, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+          <t>Oii Nayara, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
 Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
 Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
 Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
@@ -2152,14 +2152,14 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Que ótimo Cílios! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+          <t>Que ótimo Nayara! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
 👉 https://lashmenu.com/c/harmonia-rose ✨
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>Prontinho Cílios! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+          <t>Prontinho Nayara! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
 👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
 A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
 Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
@@ -2296,7 +2296,7 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Oii Cílios, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+          <t>Oii, tudo bem?, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
 Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
 Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
 Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
@@ -2304,14 +2304,14 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>Que ótimo Cílios! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+          <t>Que ótimo! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
 👉 https://lashmenu.com/c/harmonia-rose ✨
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>Prontinho Cílios! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+          <t>Prontinho! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
 👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
 A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
 Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
@@ -2440,7 +2440,7 @@
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Oii Vidal, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+          <t>Oii Priscila, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
 Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
 Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
 Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
@@ -2448,14 +2448,14 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>Que ótimo Vidal! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+          <t>Que ótimo Priscila! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
 👉 https://lashmenu.com/c/harmonia-rose ✨
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>Prontinho Vidal! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+          <t>Prontinho Priscila! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
 👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
 A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
 Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
@@ -2654,7 +2654,7 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Oii D'isanto, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+          <t>Oii D'Isanto, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
 Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
 Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
 Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
@@ -2662,14 +2662,14 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>Que ótimo D'isanto! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+          <t>Que ótimo D'Isanto! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
 👉 https://lashmenu.com/c/harmonia-rose ✨
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>Prontinho D'isanto! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+          <t>Prontinho D'Isanto! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
 👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
 A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
 Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
@@ -2732,7 +2732,7 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Oii Ynnaê, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+          <t>Oii Ynnaá, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
 Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
 Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
 Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
@@ -2740,14 +2740,14 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>Que ótimo Ynnaê! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+          <t>Que ótimo Ynnaá! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
 👉 https://lashmenu.com/c/harmonia-rose ✨
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>Prontinho Ynnaê! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+          <t>Prontinho Ynnaá! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
 👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
 A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
 Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
@@ -3020,7 +3020,7 @@
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr">
         <is>
-          <t>Oii Stúdio, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+          <t>Oii Kássia, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
 Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
 Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
 Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
@@ -3028,14 +3028,14 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>Que ótimo Stúdio! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+          <t>Que ótimo Kássia! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
 👉 https://lashmenu.com/c/harmonia-rose ✨
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>Prontinho Stúdio! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+          <t>Prontinho Kássia! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
 👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
 A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
 Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
@@ -3292,7 +3292,7 @@
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr">
         <is>
-          <t>Oii Marques, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+          <t>Oii Faby, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
 Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
 Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
 Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
@@ -3300,14 +3300,14 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>Que ótimo Marques! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+          <t>Que ótimo Faby! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
 👉 https://lashmenu.com/c/harmonia-rose ✨
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>Prontinho Marques! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+          <t>Prontinho Faby! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
 👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
 A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
 Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎
@@ -3424,7 +3424,7 @@
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr">
         <is>
-          <t>Oii Ana, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
+          <t>Oii Ana Beatriz, tudo bem? 💕 Vi o seu perfil no Google e achei os seus trabalhos de cílios simplesmente perfeitos! 😍✨
 Sei como é corrido o dia a dia e quanto tempo a gente perde no WhatsApp explicando técnicas (Fio a Fio, Volume Russo, Brasileiro) e enviando tabelas soltas... 📝📲
 Criamos o *LashMenu*, um catálogo digital interativo e super elegante para você colocar no link da bio do Instagram e mandar nas conversas, deixando seu atendimento muito mais profissional e acelerando os seus agendamentos! 💖🌸
 Posso te mandar um modelo de demonstração para você ver como fica lindo na prática? 👁️✨</t>
@@ -3432,14 +3432,14 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>Que ótimo Ana! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
+          <t>Que ótimo Ana Beatriz! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
 👉 https://lashmenu.com/c/harmonia-rose ✨
 Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>Prontinho Ana! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
+          <t>Prontinho Ana Beatriz! 🌸✨ Montei o catálogo exclusivo do seu estúdio para você dar uma olhada:
 👉 [LINK_DO_CATALOGO_PERSONALIZADO_DELA] 😍💖
 A assinatura da plataforma com suporte completo e hospedagem fica por R$ 197 no site oficial (https://lashmenu.com).
 Mas como estamos conversando diretamente por aqui no WhatsApp, conseguimos uma condição super especial de 15% de desconto via Pix: fica por apenas *R$ 167 (pagamento único sem mensalidades)*! 🎉💎

</xml_diff>

<commit_message>
feat: adiciona opcao de 3 modelos de demonstracao na mensagem 2 com Harmonia Rose em destaque
</commit_message>
<xml_diff>
--- a/Prospecção/Leads_LashDesigner_Goiania.xlsx
+++ b/Prospecção/Leads_LashDesigner_Goiania.xlsx
@@ -558,9 +558,15 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Que ótimo Edivania! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose ✨
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
+          <t>Que ótimo Edivania! 😍💖 Temos 3 modelos de catálogos incríveis para você escolher o que mais combina com a identidade do seu estúdio:
+⭐ 1. Modelo Harmonia Rosé (Nosso mais amado! 💕):
+👉 https://lashmenu.com/c/harmonia-rose ✨
+🌸 2. Modelo Clássico Rosé:
+👉 https://lashmenu.com/c/classico-rose ✨
+✨ 3. Modelo Glamour Midnight (Dark Luxo):
+👉 https://lashmenu.com/c/glamour-midnight ✨
+Dá uma olhada nesses exemplos e me fala qual estilo você mais gostou! 🥰
+Se quiser, já pode me enviar aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu monto a versão personalizada do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -636,9 +642,15 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Que ótimo Layfer! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose ✨
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
+          <t>Que ótimo Layfer! 😍💖 Temos 3 modelos de catálogos incríveis para você escolher o que mais combina com a identidade do seu estúdio:
+⭐ 1. Modelo Harmonia Rosé (Nosso mais amado! 💕):
+👉 https://lashmenu.com/c/harmonia-rose ✨
+🌸 2. Modelo Clássico Rosé:
+👉 https://lashmenu.com/c/classico-rose ✨
+✨ 3. Modelo Glamour Midnight (Dark Luxo):
+👉 https://lashmenu.com/c/glamour-midnight ✨
+Dá uma olhada nesses exemplos e me fala qual estilo você mais gostou! 🥰
+Se quiser, já pode me enviar aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu monto a versão personalizada do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -710,9 +722,15 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Que ótimo Larissa! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose ✨
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
+          <t>Que ótimo Larissa! 😍💖 Temos 3 modelos de catálogos incríveis para você escolher o que mais combina com a identidade do seu estúdio:
+⭐ 1. Modelo Harmonia Rosé (Nosso mais amado! 💕):
+👉 https://lashmenu.com/c/harmonia-rose ✨
+🌸 2. Modelo Clássico Rosé:
+👉 https://lashmenu.com/c/classico-rose ✨
+✨ 3. Modelo Glamour Midnight (Dark Luxo):
+👉 https://lashmenu.com/c/glamour-midnight ✨
+Dá uma olhada nesses exemplos e me fala qual estilo você mais gostou! 🥰
+Se quiser, já pode me enviar aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu monto a versão personalizada do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -784,9 +802,15 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Que ótimo Leticia! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose ✨
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
+          <t>Que ótimo Leticia! 😍💖 Temos 3 modelos de catálogos incríveis para você escolher o que mais combina com a identidade do seu estúdio:
+⭐ 1. Modelo Harmonia Rosé (Nosso mais amado! 💕):
+👉 https://lashmenu.com/c/harmonia-rose ✨
+🌸 2. Modelo Clássico Rosé:
+👉 https://lashmenu.com/c/classico-rose ✨
+✨ 3. Modelo Glamour Midnight (Dark Luxo):
+👉 https://lashmenu.com/c/glamour-midnight ✨
+Dá uma olhada nesses exemplos e me fala qual estilo você mais gostou! 🥰
+Se quiser, já pode me enviar aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu monto a versão personalizada do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -858,9 +882,15 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Que ótimo Poliana! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose ✨
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
+          <t>Que ótimo Poliana! 😍💖 Temos 3 modelos de catálogos incríveis para você escolher o que mais combina com a identidade do seu estúdio:
+⭐ 1. Modelo Harmonia Rosé (Nosso mais amado! 💕):
+👉 https://lashmenu.com/c/harmonia-rose ✨
+🌸 2. Modelo Clássico Rosé:
+👉 https://lashmenu.com/c/classico-rose ✨
+✨ 3. Modelo Glamour Midnight (Dark Luxo):
+👉 https://lashmenu.com/c/glamour-midnight ✨
+Dá uma olhada nesses exemplos e me fala qual estilo você mais gostou! 🥰
+Se quiser, já pode me enviar aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu monto a versão personalizada do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -936,9 +966,15 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Que ótimo Tanielly! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose ✨
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
+          <t>Que ótimo Tanielly! 😍💖 Temos 3 modelos de catálogos incríveis para você escolher o que mais combina com a identidade do seu estúdio:
+⭐ 1. Modelo Harmonia Rosé (Nosso mais amado! 💕):
+👉 https://lashmenu.com/c/harmonia-rose ✨
+🌸 2. Modelo Clássico Rosé:
+👉 https://lashmenu.com/c/classico-rose ✨
+✨ 3. Modelo Glamour Midnight (Dark Luxo):
+👉 https://lashmenu.com/c/glamour-midnight ✨
+Dá uma olhada nesses exemplos e me fala qual estilo você mais gostou! 🥰
+Se quiser, já pode me enviar aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu monto a versão personalizada do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1010,9 +1046,15 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Que ótimo Serena! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose ✨
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
+          <t>Que ótimo Serena! 😍💖 Temos 3 modelos de catálogos incríveis para você escolher o que mais combina com a identidade do seu estúdio:
+⭐ 1. Modelo Harmonia Rosé (Nosso mais amado! 💕):
+👉 https://lashmenu.com/c/harmonia-rose ✨
+🌸 2. Modelo Clássico Rosé:
+👉 https://lashmenu.com/c/classico-rose ✨
+✨ 3. Modelo Glamour Midnight (Dark Luxo):
+👉 https://lashmenu.com/c/glamour-midnight ✨
+Dá uma olhada nesses exemplos e me fala qual estilo você mais gostou! 🥰
+Se quiser, já pode me enviar aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu monto a versão personalizada do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1088,9 +1130,15 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Que ótimo Cinthya! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose ✨
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
+          <t>Que ótimo Cinthya! 😍💖 Temos 3 modelos de catálogos incríveis para você escolher o que mais combina com a identidade do seu estúdio:
+⭐ 1. Modelo Harmonia Rosé (Nosso mais amado! 💕):
+👉 https://lashmenu.com/c/harmonia-rose ✨
+🌸 2. Modelo Clássico Rosé:
+👉 https://lashmenu.com/c/classico-rose ✨
+✨ 3. Modelo Glamour Midnight (Dark Luxo):
+👉 https://lashmenu.com/c/glamour-midnight ✨
+Dá uma olhada nesses exemplos e me fala qual estilo você mais gostou! 🥰
+Se quiser, já pode me enviar aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu monto a versão personalizada do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1166,9 +1214,15 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Que ótimo Milenne! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose ✨
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
+          <t>Que ótimo Milenne! 😍💖 Temos 3 modelos de catálogos incríveis para você escolher o que mais combina com a identidade do seu estúdio:
+⭐ 1. Modelo Harmonia Rosé (Nosso mais amado! 💕):
+👉 https://lashmenu.com/c/harmonia-rose ✨
+🌸 2. Modelo Clássico Rosé:
+👉 https://lashmenu.com/c/classico-rose ✨
+✨ 3. Modelo Glamour Midnight (Dark Luxo):
+👉 https://lashmenu.com/c/glamour-midnight ✨
+Dá uma olhada nesses exemplos e me fala qual estilo você mais gostou! 🥰
+Se quiser, já pode me enviar aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu monto a versão personalizada do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1244,9 +1298,15 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Que ótimo Brunna! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose ✨
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
+          <t>Que ótimo Brunna! 😍💖 Temos 3 modelos de catálogos incríveis para você escolher o que mais combina com a identidade do seu estúdio:
+⭐ 1. Modelo Harmonia Rosé (Nosso mais amado! 💕):
+👉 https://lashmenu.com/c/harmonia-rose ✨
+🌸 2. Modelo Clássico Rosé:
+👉 https://lashmenu.com/c/classico-rose ✨
+✨ 3. Modelo Glamour Midnight (Dark Luxo):
+👉 https://lashmenu.com/c/glamour-midnight ✨
+Dá uma olhada nesses exemplos e me fala qual estilo você mais gostou! 🥰
+Se quiser, já pode me enviar aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu monto a versão personalizada do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1322,9 +1382,15 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Que ótimo Bella! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose ✨
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
+          <t>Que ótimo Bella! 😍💖 Temos 3 modelos de catálogos incríveis para você escolher o que mais combina com a identidade do seu estúdio:
+⭐ 1. Modelo Harmonia Rosé (Nosso mais amado! 💕):
+👉 https://lashmenu.com/c/harmonia-rose ✨
+🌸 2. Modelo Clássico Rosé:
+👉 https://lashmenu.com/c/classico-rose ✨
+✨ 3. Modelo Glamour Midnight (Dark Luxo):
+👉 https://lashmenu.com/c/glamour-midnight ✨
+Dá uma olhada nesses exemplos e me fala qual estilo você mais gostou! 🥰
+Se quiser, já pode me enviar aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu monto a versão personalizada do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1400,9 +1466,15 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>Que ótimo Maria Eugênia! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose ✨
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
+          <t>Que ótimo Maria Eugênia! 😍💖 Temos 3 modelos de catálogos incríveis para você escolher o que mais combina com a identidade do seu estúdio:
+⭐ 1. Modelo Harmonia Rosé (Nosso mais amado! 💕):
+👉 https://lashmenu.com/c/harmonia-rose ✨
+🌸 2. Modelo Clássico Rosé:
+👉 https://lashmenu.com/c/classico-rose ✨
+✨ 3. Modelo Glamour Midnight (Dark Luxo):
+👉 https://lashmenu.com/c/glamour-midnight ✨
+Dá uma olhada nesses exemplos e me fala qual estilo você mais gostou! 🥰
+Se quiser, já pode me enviar aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu monto a versão personalizada do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1478,9 +1550,15 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Que ótimo Mariane! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose ✨
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
+          <t>Que ótimo Mariane! 😍💖 Temos 3 modelos de catálogos incríveis para você escolher o que mais combina com a identidade do seu estúdio:
+⭐ 1. Modelo Harmonia Rosé (Nosso mais amado! 💕):
+👉 https://lashmenu.com/c/harmonia-rose ✨
+🌸 2. Modelo Clássico Rosé:
+👉 https://lashmenu.com/c/classico-rose ✨
+✨ 3. Modelo Glamour Midnight (Dark Luxo):
+👉 https://lashmenu.com/c/glamour-midnight ✨
+Dá uma olhada nesses exemplos e me fala qual estilo você mais gostou! 🥰
+Se quiser, já pode me enviar aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu monto a versão personalizada do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1556,9 +1634,15 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Que ótimo Isabela! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose ✨
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
+          <t>Que ótimo Isabela! 😍💖 Temos 3 modelos de catálogos incríveis para você escolher o que mais combina com a identidade do seu estúdio:
+⭐ 1. Modelo Harmonia Rosé (Nosso mais amado! 💕):
+👉 https://lashmenu.com/c/harmonia-rose ✨
+🌸 2. Modelo Clássico Rosé:
+👉 https://lashmenu.com/c/classico-rose ✨
+✨ 3. Modelo Glamour Midnight (Dark Luxo):
+👉 https://lashmenu.com/c/glamour-midnight ✨
+Dá uma olhada nesses exemplos e me fala qual estilo você mais gostou! 🥰
+Se quiser, já pode me enviar aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu monto a versão personalizada do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1634,9 +1718,15 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Que ótimo Déborah! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose ✨
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
+          <t>Que ótimo Déborah! 😍💖 Temos 3 modelos de catálogos incríveis para você escolher o que mais combina com a identidade do seu estúdio:
+⭐ 1. Modelo Harmonia Rosé (Nosso mais amado! 💕):
+👉 https://lashmenu.com/c/harmonia-rose ✨
+🌸 2. Modelo Clássico Rosé:
+👉 https://lashmenu.com/c/classico-rose ✨
+✨ 3. Modelo Glamour Midnight (Dark Luxo):
+👉 https://lashmenu.com/c/glamour-midnight ✨
+Dá uma olhada nesses exemplos e me fala qual estilo você mais gostou! 🥰
+Se quiser, já pode me enviar aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu monto a versão personalizada do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -1712,9 +1802,15 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Que ótimo Yara! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose ✨
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
+          <t>Que ótimo Yara! 😍💖 Temos 3 modelos de catálogos incríveis para você escolher o que mais combina com a identidade do seu estúdio:
+⭐ 1. Modelo Harmonia Rosé (Nosso mais amado! 💕):
+👉 https://lashmenu.com/c/harmonia-rose ✨
+🌸 2. Modelo Clássico Rosé:
+👉 https://lashmenu.com/c/classico-rose ✨
+✨ 3. Modelo Glamour Midnight (Dark Luxo):
+👉 https://lashmenu.com/c/glamour-midnight ✨
+Dá uma olhada nesses exemplos e me fala qual estilo você mais gostou! 🥰
+Se quiser, já pode me enviar aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu monto a versão personalizada do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -1786,9 +1882,15 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Que ótimo Kathellem! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose ✨
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
+          <t>Que ótimo Kathellem! 😍💖 Temos 3 modelos de catálogos incríveis para você escolher o que mais combina com a identidade do seu estúdio:
+⭐ 1. Modelo Harmonia Rosé (Nosso mais amado! 💕):
+👉 https://lashmenu.com/c/harmonia-rose ✨
+🌸 2. Modelo Clássico Rosé:
+👉 https://lashmenu.com/c/classico-rose ✨
+✨ 3. Modelo Glamour Midnight (Dark Luxo):
+👉 https://lashmenu.com/c/glamour-midnight ✨
+Dá uma olhada nesses exemplos e me fala qual estilo você mais gostou! 🥰
+Se quiser, já pode me enviar aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu monto a versão personalizada do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -1860,9 +1962,15 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Que ótimo Lollys! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose ✨
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
+          <t>Que ótimo Lollys! 😍💖 Temos 3 modelos de catálogos incríveis para você escolher o que mais combina com a identidade do seu estúdio:
+⭐ 1. Modelo Harmonia Rosé (Nosso mais amado! 💕):
+👉 https://lashmenu.com/c/harmonia-rose ✨
+🌸 2. Modelo Clássico Rosé:
+👉 https://lashmenu.com/c/classico-rose ✨
+✨ 3. Modelo Glamour Midnight (Dark Luxo):
+👉 https://lashmenu.com/c/glamour-midnight ✨
+Dá uma olhada nesses exemplos e me fala qual estilo você mais gostou! 🥰
+Se quiser, já pode me enviar aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu monto a versão personalizada do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -1930,9 +2038,15 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Que ótimo Ariana! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose ✨
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
+          <t>Que ótimo Ariana! 😍💖 Temos 3 modelos de catálogos incríveis para você escolher o que mais combina com a identidade do seu estúdio:
+⭐ 1. Modelo Harmonia Rosé (Nosso mais amado! 💕):
+👉 https://lashmenu.com/c/harmonia-rose ✨
+🌸 2. Modelo Clássico Rosé:
+👉 https://lashmenu.com/c/classico-rose ✨
+✨ 3. Modelo Glamour Midnight (Dark Luxo):
+👉 https://lashmenu.com/c/glamour-midnight ✨
+Dá uma olhada nesses exemplos e me fala qual estilo você mais gostou! 🥰
+Se quiser, já pode me enviar aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu monto a versão personalizada do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -2000,9 +2114,15 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Que ótimo! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose ✨
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
+          <t>Que ótimo! 😍💖 Temos 3 modelos de catálogos incríveis para você escolher o que mais combina com a identidade do seu estúdio:
+⭐ 1. Modelo Harmonia Rosé (Nosso mais amado! 💕):
+👉 https://lashmenu.com/c/harmonia-rose ✨
+🌸 2. Modelo Clássico Rosé:
+👉 https://lashmenu.com/c/classico-rose ✨
+✨ 3. Modelo Glamour Midnight (Dark Luxo):
+👉 https://lashmenu.com/c/glamour-midnight ✨
+Dá uma olhada nesses exemplos e me fala qual estilo você mais gostou! 🥰
+Se quiser, já pode me enviar aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu monto a versão personalizada do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -2078,9 +2198,15 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Que ótimo Elaíne! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose ✨
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
+          <t>Que ótimo Elaíne! 😍💖 Temos 3 modelos de catálogos incríveis para você escolher o que mais combina com a identidade do seu estúdio:
+⭐ 1. Modelo Harmonia Rosé (Nosso mais amado! 💕):
+👉 https://lashmenu.com/c/harmonia-rose ✨
+🌸 2. Modelo Clássico Rosé:
+👉 https://lashmenu.com/c/classico-rose ✨
+✨ 3. Modelo Glamour Midnight (Dark Luxo):
+👉 https://lashmenu.com/c/glamour-midnight ✨
+Dá uma olhada nesses exemplos e me fala qual estilo você mais gostou! 🥰
+Se quiser, já pode me enviar aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu monto a versão personalizada do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -2152,9 +2278,15 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Que ótimo Nayara! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose ✨
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
+          <t>Que ótimo Nayara! 😍💖 Temos 3 modelos de catálogos incríveis para você escolher o que mais combina com a identidade do seu estúdio:
+⭐ 1. Modelo Harmonia Rosé (Nosso mais amado! 💕):
+👉 https://lashmenu.com/c/harmonia-rose ✨
+🌸 2. Modelo Clássico Rosé:
+👉 https://lashmenu.com/c/classico-rose ✨
+✨ 3. Modelo Glamour Midnight (Dark Luxo):
+👉 https://lashmenu.com/c/glamour-midnight ✨
+Dá uma olhada nesses exemplos e me fala qual estilo você mais gostou! 🥰
+Se quiser, já pode me enviar aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu monto a versão personalizada do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2230,9 +2362,15 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Que ótimo Joana! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose ✨
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
+          <t>Que ótimo Joana! 😍💖 Temos 3 modelos de catálogos incríveis para você escolher o que mais combina com a identidade do seu estúdio:
+⭐ 1. Modelo Harmonia Rosé (Nosso mais amado! 💕):
+👉 https://lashmenu.com/c/harmonia-rose ✨
+🌸 2. Modelo Clássico Rosé:
+👉 https://lashmenu.com/c/classico-rose ✨
+✨ 3. Modelo Glamour Midnight (Dark Luxo):
+👉 https://lashmenu.com/c/glamour-midnight ✨
+Dá uma olhada nesses exemplos e me fala qual estilo você mais gostou! 🥰
+Se quiser, já pode me enviar aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu monto a versão personalizada do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -2304,9 +2442,15 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>Que ótimo! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose ✨
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
+          <t>Que ótimo! 😍💖 Temos 3 modelos de catálogos incríveis para você escolher o que mais combina com a identidade do seu estúdio:
+⭐ 1. Modelo Harmonia Rosé (Nosso mais amado! 💕):
+👉 https://lashmenu.com/c/harmonia-rose ✨
+🌸 2. Modelo Clássico Rosé:
+👉 https://lashmenu.com/c/classico-rose ✨
+✨ 3. Modelo Glamour Midnight (Dark Luxo):
+👉 https://lashmenu.com/c/glamour-midnight ✨
+Dá uma olhada nesses exemplos e me fala qual estilo você mais gostou! 🥰
+Se quiser, já pode me enviar aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu monto a versão personalizada do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -2378,9 +2522,15 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Que ótimo Katyane! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose ✨
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
+          <t>Que ótimo Katyane! 😍💖 Temos 3 modelos de catálogos incríveis para você escolher o que mais combina com a identidade do seu estúdio:
+⭐ 1. Modelo Harmonia Rosé (Nosso mais amado! 💕):
+👉 https://lashmenu.com/c/harmonia-rose ✨
+🌸 2. Modelo Clássico Rosé:
+👉 https://lashmenu.com/c/classico-rose ✨
+✨ 3. Modelo Glamour Midnight (Dark Luxo):
+👉 https://lashmenu.com/c/glamour-midnight ✨
+Dá uma olhada nesses exemplos e me fala qual estilo você mais gostou! 🥰
+Se quiser, já pode me enviar aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu monto a versão personalizada do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -2448,9 +2598,15 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>Que ótimo Priscila! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose ✨
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
+          <t>Que ótimo Priscila! 😍💖 Temos 3 modelos de catálogos incríveis para você escolher o que mais combina com a identidade do seu estúdio:
+⭐ 1. Modelo Harmonia Rosé (Nosso mais amado! 💕):
+👉 https://lashmenu.com/c/harmonia-rose ✨
+🌸 2. Modelo Clássico Rosé:
+👉 https://lashmenu.com/c/classico-rose ✨
+✨ 3. Modelo Glamour Midnight (Dark Luxo):
+👉 https://lashmenu.com/c/glamour-midnight ✨
+Dá uma olhada nesses exemplos e me fala qual estilo você mais gostou! 🥰
+Se quiser, já pode me enviar aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu monto a versão personalizada do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -2518,9 +2674,15 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>Que ótimo Crys! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose ✨
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
+          <t>Que ótimo Crys! 😍💖 Temos 3 modelos de catálogos incríveis para você escolher o que mais combina com a identidade do seu estúdio:
+⭐ 1. Modelo Harmonia Rosé (Nosso mais amado! 💕):
+👉 https://lashmenu.com/c/harmonia-rose ✨
+🌸 2. Modelo Clássico Rosé:
+👉 https://lashmenu.com/c/classico-rose ✨
+✨ 3. Modelo Glamour Midnight (Dark Luxo):
+👉 https://lashmenu.com/c/glamour-midnight ✨
+Dá uma olhada nesses exemplos e me fala qual estilo você mais gostou! 🥰
+Se quiser, já pode me enviar aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu monto a versão personalizada do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -2588,9 +2750,15 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>Que ótimo Aliany! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose ✨
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
+          <t>Que ótimo Aliany! 😍💖 Temos 3 modelos de catálogos incríveis para você escolher o que mais combina com a identidade do seu estúdio:
+⭐ 1. Modelo Harmonia Rosé (Nosso mais amado! 💕):
+👉 https://lashmenu.com/c/harmonia-rose ✨
+🌸 2. Modelo Clássico Rosé:
+👉 https://lashmenu.com/c/classico-rose ✨
+✨ 3. Modelo Glamour Midnight (Dark Luxo):
+👉 https://lashmenu.com/c/glamour-midnight ✨
+Dá uma olhada nesses exemplos e me fala qual estilo você mais gostou! 🥰
+Se quiser, já pode me enviar aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu monto a versão personalizada do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -2662,9 +2830,15 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>Que ótimo D'Isanto! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose ✨
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
+          <t>Que ótimo D'Isanto! 😍💖 Temos 3 modelos de catálogos incríveis para você escolher o que mais combina com a identidade do seu estúdio:
+⭐ 1. Modelo Harmonia Rosé (Nosso mais amado! 💕):
+👉 https://lashmenu.com/c/harmonia-rose ✨
+🌸 2. Modelo Clássico Rosé:
+👉 https://lashmenu.com/c/classico-rose ✨
+✨ 3. Modelo Glamour Midnight (Dark Luxo):
+👉 https://lashmenu.com/c/glamour-midnight ✨
+Dá uma olhada nesses exemplos e me fala qual estilo você mais gostou! 🥰
+Se quiser, já pode me enviar aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu monto a versão personalizada do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -2740,9 +2914,15 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>Que ótimo Ynnaá! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose ✨
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
+          <t>Que ótimo Ynnaá! 😍💖 Temos 3 modelos de catálogos incríveis para você escolher o que mais combina com a identidade do seu estúdio:
+⭐ 1. Modelo Harmonia Rosé (Nosso mais amado! 💕):
+👉 https://lashmenu.com/c/harmonia-rose ✨
+🌸 2. Modelo Clássico Rosé:
+👉 https://lashmenu.com/c/classico-rose ✨
+✨ 3. Modelo Glamour Midnight (Dark Luxo):
+👉 https://lashmenu.com/c/glamour-midnight ✨
+Dá uma olhada nesses exemplos e me fala qual estilo você mais gostou! 🥰
+Se quiser, já pode me enviar aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu monto a versão personalizada do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -2818,9 +2998,15 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>Que ótimo Tiffany! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose ✨
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
+          <t>Que ótimo Tiffany! 😍💖 Temos 3 modelos de catálogos incríveis para você escolher o que mais combina com a identidade do seu estúdio:
+⭐ 1. Modelo Harmonia Rosé (Nosso mais amado! 💕):
+👉 https://lashmenu.com/c/harmonia-rose ✨
+🌸 2. Modelo Clássico Rosé:
+👉 https://lashmenu.com/c/classico-rose ✨
+✨ 3. Modelo Glamour Midnight (Dark Luxo):
+👉 https://lashmenu.com/c/glamour-midnight ✨
+Dá uma olhada nesses exemplos e me fala qual estilo você mais gostou! 🥰
+Se quiser, já pode me enviar aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu monto a versão personalizada do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -2888,9 +3074,15 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>Que ótimo Luana! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose ✨
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
+          <t>Que ótimo Luana! 😍💖 Temos 3 modelos de catálogos incríveis para você escolher o que mais combina com a identidade do seu estúdio:
+⭐ 1. Modelo Harmonia Rosé (Nosso mais amado! 💕):
+👉 https://lashmenu.com/c/harmonia-rose ✨
+🌸 2. Modelo Clássico Rosé:
+👉 https://lashmenu.com/c/classico-rose ✨
+✨ 3. Modelo Glamour Midnight (Dark Luxo):
+👉 https://lashmenu.com/c/glamour-midnight ✨
+Dá uma olhada nesses exemplos e me fala qual estilo você mais gostou! 🥰
+Se quiser, já pode me enviar aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu monto a versão personalizada do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -2958,9 +3150,15 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>Que ótimo Maiza! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose ✨
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
+          <t>Que ótimo Maiza! 😍💖 Temos 3 modelos de catálogos incríveis para você escolher o que mais combina com a identidade do seu estúdio:
+⭐ 1. Modelo Harmonia Rosé (Nosso mais amado! 💕):
+👉 https://lashmenu.com/c/harmonia-rose ✨
+🌸 2. Modelo Clássico Rosé:
+👉 https://lashmenu.com/c/classico-rose ✨
+✨ 3. Modelo Glamour Midnight (Dark Luxo):
+👉 https://lashmenu.com/c/glamour-midnight ✨
+Dá uma olhada nesses exemplos e me fala qual estilo você mais gostou! 🥰
+Se quiser, já pode me enviar aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu monto a versão personalizada do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -3028,9 +3226,15 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>Que ótimo Kássia! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose ✨
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
+          <t>Que ótimo Kássia! 😍💖 Temos 3 modelos de catálogos incríveis para você escolher o que mais combina com a identidade do seu estúdio:
+⭐ 1. Modelo Harmonia Rosé (Nosso mais amado! 💕):
+👉 https://lashmenu.com/c/harmonia-rose ✨
+🌸 2. Modelo Clássico Rosé:
+👉 https://lashmenu.com/c/classico-rose ✨
+✨ 3. Modelo Glamour Midnight (Dark Luxo):
+👉 https://lashmenu.com/c/glamour-midnight ✨
+Dá uma olhada nesses exemplos e me fala qual estilo você mais gostou! 🥰
+Se quiser, já pode me enviar aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu monto a versão personalizada do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -3090,9 +3294,15 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>Que ótimo Jéssica! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose ✨
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
+          <t>Que ótimo Jéssica! 😍💖 Temos 3 modelos de catálogos incríveis para você escolher o que mais combina com a identidade do seu estúdio:
+⭐ 1. Modelo Harmonia Rosé (Nosso mais amado! 💕):
+👉 https://lashmenu.com/c/harmonia-rose ✨
+🌸 2. Modelo Clássico Rosé:
+👉 https://lashmenu.com/c/classico-rose ✨
+✨ 3. Modelo Glamour Midnight (Dark Luxo):
+👉 https://lashmenu.com/c/glamour-midnight ✨
+Dá uma olhada nesses exemplos e me fala qual estilo você mais gostou! 🥰
+Se quiser, já pode me enviar aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu monto a versão personalizada do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -3160,9 +3370,15 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>Que ótimo Carvalho! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose ✨
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
+          <t>Que ótimo Carvalho! 😍💖 Temos 3 modelos de catálogos incríveis para você escolher o que mais combina com a identidade do seu estúdio:
+⭐ 1. Modelo Harmonia Rosé (Nosso mais amado! 💕):
+👉 https://lashmenu.com/c/harmonia-rose ✨
+🌸 2. Modelo Clássico Rosé:
+👉 https://lashmenu.com/c/classico-rose ✨
+✨ 3. Modelo Glamour Midnight (Dark Luxo):
+👉 https://lashmenu.com/c/glamour-midnight ✨
+Dá uma olhada nesses exemplos e me fala qual estilo você mais gostou! 🥰
+Se quiser, já pode me enviar aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu monto a versão personalizada do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -3230,9 +3446,15 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>Que ótimo Lanna! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose ✨
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
+          <t>Que ótimo Lanna! 😍💖 Temos 3 modelos de catálogos incríveis para você escolher o que mais combina com a identidade do seu estúdio:
+⭐ 1. Modelo Harmonia Rosé (Nosso mais amado! 💕):
+👉 https://lashmenu.com/c/harmonia-rose ✨
+🌸 2. Modelo Clássico Rosé:
+👉 https://lashmenu.com/c/classico-rose ✨
+✨ 3. Modelo Glamour Midnight (Dark Luxo):
+👉 https://lashmenu.com/c/glamour-midnight ✨
+Dá uma olhada nesses exemplos e me fala qual estilo você mais gostou! 🥰
+Se quiser, já pode me enviar aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu monto a versão personalizada do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -3300,9 +3522,15 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>Que ótimo Faby! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose ✨
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
+          <t>Que ótimo Faby! 😍💖 Temos 3 modelos de catálogos incríveis para você escolher o que mais combina com a identidade do seu estúdio:
+⭐ 1. Modelo Harmonia Rosé (Nosso mais amado! 💕):
+👉 https://lashmenu.com/c/harmonia-rose ✨
+🌸 2. Modelo Clássico Rosé:
+👉 https://lashmenu.com/c/classico-rose ✨
+✨ 3. Modelo Glamour Midnight (Dark Luxo):
+👉 https://lashmenu.com/c/glamour-midnight ✨
+Dá uma olhada nesses exemplos e me fala qual estilo você mais gostou! 🥰
+Se quiser, já pode me enviar aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu monto a versão personalizada do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -3370,9 +3598,15 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>Que ótimo Sara! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose ✨
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
+          <t>Que ótimo Sara! 😍💖 Temos 3 modelos de catálogos incríveis para você escolher o que mais combina com a identidade do seu estúdio:
+⭐ 1. Modelo Harmonia Rosé (Nosso mais amado! 💕):
+👉 https://lashmenu.com/c/harmonia-rose ✨
+🌸 2. Modelo Clássico Rosé:
+👉 https://lashmenu.com/c/classico-rose ✨
+✨ 3. Modelo Glamour Midnight (Dark Luxo):
+👉 https://lashmenu.com/c/glamour-midnight ✨
+Dá uma olhada nesses exemplos e me fala qual estilo você mais gostou! 🥰
+Se quiser, já pode me enviar aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu monto a versão personalizada do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
@@ -3432,9 +3666,15 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>Que ótimo Ana Beatriz! 😍💖 Segue o link de um modelo pronto para você testar a experiência como se fosse sua cliente:
-👉 https://lashmenu.com/c/harmonia-rose ✨
-Se você gostar da estrutura, me envia aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu já monto a versão exclusiva do seu estúdio para você ver na prática! 🌸📲</t>
+          <t>Que ótimo Ana Beatriz! 😍💖 Temos 3 modelos de catálogos incríveis para você escolher o que mais combina com a identidade do seu estúdio:
+⭐ 1. Modelo Harmonia Rosé (Nosso mais amado! 💕):
+👉 https://lashmenu.com/c/harmonia-rose ✨
+🌸 2. Modelo Clássico Rosé:
+👉 https://lashmenu.com/c/classico-rose ✨
+✨ 3. Modelo Glamour Midnight (Dark Luxo):
+👉 https://lashmenu.com/c/glamour-midnight ✨
+Dá uma olhada nesses exemplos e me fala qual estilo você mais gostou! 🥰
+Se quiser, já pode me enviar aqui uma foto ou lista dos seus procedimentos com os preços atuais que eu monto a versão personalizada do seu estúdio para você ver na prática! 🌸📲</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">

</xml_diff>